<commit_message>
fix bug ground module
</commit_message>
<xml_diff>
--- a/src/main/resources/static/Sample_Excel_Import_Asset.xlsx
+++ b/src/main/resources/static/Sample_Excel_Import_Asset.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\Zalo Received Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hieux\Desktop\Projects\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1463C2-6CAF-42F4-80D7-DB5F61848DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A54E6F-78A5-42B1-8F2F-FC232440773D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="105" yWindow="240" windowWidth="28695" windowHeight="15240" activeTab="1" xr2:uid="{71050258-D013-4370-AEE7-AC2797CFA723}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{71050258-D013-4370-AEE7-AC2797CFA723}"/>
   </bookViews>
   <sheets>
     <sheet name="ImportAsset" sheetId="1" r:id="rId1"/>
-    <sheet name="Huongdannhapthongtin" sheetId="2" r:id="rId2"/>
+    <sheet name="Hướng dẫn nhập thông tin" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="269">
   <si>
     <t>Thông tin chung</t>
   </si>
@@ -1028,9 +1028,6 @@
   <si>
     <t>Ngân sách Xã</t>
   </si>
-  <si>
-    <t>2;3</t>
-  </si>
 </sst>
 </file>
 
@@ -1610,10 +1607,76 @@
     <xf numFmtId="0" fontId="3" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="15" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="19" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="19" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1673,9 +1736,6 @@
     <xf numFmtId="49" fontId="2" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1685,67 +1745,79 @@
     <xf numFmtId="49" fontId="1" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="15" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="19" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="19" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1799,18 +1871,6 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1824,69 +1884,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2248,378 +2245,378 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:146" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="90" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="71" t="s">
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="92"/>
+      <c r="Q1" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="72"/>
-      <c r="S1" s="72"/>
-      <c r="T1" s="72"/>
-      <c r="U1" s="72"/>
-      <c r="V1" s="72"/>
-      <c r="W1" s="72"/>
-      <c r="X1" s="72"/>
-      <c r="Y1" s="72"/>
-      <c r="Z1" s="72"/>
-      <c r="AA1" s="72"/>
-      <c r="AB1" s="72"/>
-      <c r="AC1" s="72"/>
-      <c r="AD1" s="72"/>
-      <c r="AE1" s="72"/>
-      <c r="AF1" s="72"/>
-      <c r="AG1" s="72"/>
-      <c r="AH1" s="72"/>
-      <c r="AI1" s="72"/>
-      <c r="AJ1" s="72"/>
-      <c r="AK1" s="72"/>
-      <c r="AL1" s="72"/>
-      <c r="AM1" s="72"/>
-      <c r="AN1" s="72"/>
-      <c r="AO1" s="72"/>
-      <c r="AP1" s="72"/>
-      <c r="AQ1" s="72"/>
-      <c r="AR1" s="72"/>
-      <c r="AS1" s="72"/>
-      <c r="AT1" s="72"/>
-      <c r="AU1" s="72"/>
-      <c r="AV1" s="72"/>
-      <c r="AW1" s="72"/>
-      <c r="AX1" s="72"/>
-      <c r="AY1" s="72"/>
-      <c r="AZ1" s="72"/>
-      <c r="BA1" s="72"/>
-      <c r="BB1" s="72"/>
-      <c r="BC1" s="72"/>
-      <c r="BD1" s="72"/>
-      <c r="BE1" s="72"/>
-      <c r="BF1" s="72"/>
-      <c r="BG1" s="72"/>
-      <c r="BH1" s="72"/>
-      <c r="BI1" s="72"/>
-      <c r="BJ1" s="72"/>
-      <c r="BK1" s="72"/>
-      <c r="BL1" s="72"/>
-      <c r="BM1" s="72"/>
-      <c r="BN1" s="72"/>
-      <c r="BO1" s="72"/>
-      <c r="BP1" s="72"/>
-      <c r="BQ1" s="72"/>
-      <c r="BR1" s="72"/>
-      <c r="BS1" s="72"/>
-      <c r="BT1" s="72"/>
-      <c r="BU1" s="72"/>
-      <c r="BV1" s="72"/>
-      <c r="BW1" s="72"/>
-      <c r="BX1" s="72"/>
-      <c r="BY1" s="72"/>
-      <c r="BZ1" s="72"/>
-      <c r="CA1" s="72"/>
-      <c r="CB1" s="72"/>
-      <c r="CC1" s="72"/>
-      <c r="CD1" s="72"/>
-      <c r="CE1" s="72"/>
-      <c r="CF1" s="72"/>
-      <c r="CG1" s="72"/>
-      <c r="CH1" s="72"/>
-      <c r="CI1" s="72"/>
-      <c r="CJ1" s="72"/>
-      <c r="CK1" s="72"/>
-      <c r="CL1" s="72"/>
-      <c r="CM1" s="72"/>
-      <c r="CN1" s="72"/>
-      <c r="CO1" s="73"/>
-      <c r="CP1" s="74" t="s">
+      <c r="R1" s="94"/>
+      <c r="S1" s="94"/>
+      <c r="T1" s="94"/>
+      <c r="U1" s="94"/>
+      <c r="V1" s="94"/>
+      <c r="W1" s="94"/>
+      <c r="X1" s="94"/>
+      <c r="Y1" s="94"/>
+      <c r="Z1" s="94"/>
+      <c r="AA1" s="94"/>
+      <c r="AB1" s="94"/>
+      <c r="AC1" s="94"/>
+      <c r="AD1" s="94"/>
+      <c r="AE1" s="94"/>
+      <c r="AF1" s="94"/>
+      <c r="AG1" s="94"/>
+      <c r="AH1" s="94"/>
+      <c r="AI1" s="94"/>
+      <c r="AJ1" s="94"/>
+      <c r="AK1" s="94"/>
+      <c r="AL1" s="94"/>
+      <c r="AM1" s="94"/>
+      <c r="AN1" s="94"/>
+      <c r="AO1" s="94"/>
+      <c r="AP1" s="94"/>
+      <c r="AQ1" s="94"/>
+      <c r="AR1" s="94"/>
+      <c r="AS1" s="94"/>
+      <c r="AT1" s="94"/>
+      <c r="AU1" s="94"/>
+      <c r="AV1" s="94"/>
+      <c r="AW1" s="94"/>
+      <c r="AX1" s="94"/>
+      <c r="AY1" s="94"/>
+      <c r="AZ1" s="94"/>
+      <c r="BA1" s="94"/>
+      <c r="BB1" s="94"/>
+      <c r="BC1" s="94"/>
+      <c r="BD1" s="94"/>
+      <c r="BE1" s="94"/>
+      <c r="BF1" s="94"/>
+      <c r="BG1" s="94"/>
+      <c r="BH1" s="94"/>
+      <c r="BI1" s="94"/>
+      <c r="BJ1" s="94"/>
+      <c r="BK1" s="94"/>
+      <c r="BL1" s="94"/>
+      <c r="BM1" s="94"/>
+      <c r="BN1" s="94"/>
+      <c r="BO1" s="94"/>
+      <c r="BP1" s="94"/>
+      <c r="BQ1" s="94"/>
+      <c r="BR1" s="94"/>
+      <c r="BS1" s="94"/>
+      <c r="BT1" s="94"/>
+      <c r="BU1" s="94"/>
+      <c r="BV1" s="94"/>
+      <c r="BW1" s="94"/>
+      <c r="BX1" s="94"/>
+      <c r="BY1" s="94"/>
+      <c r="BZ1" s="94"/>
+      <c r="CA1" s="94"/>
+      <c r="CB1" s="94"/>
+      <c r="CC1" s="94"/>
+      <c r="CD1" s="94"/>
+      <c r="CE1" s="94"/>
+      <c r="CF1" s="94"/>
+      <c r="CG1" s="94"/>
+      <c r="CH1" s="94"/>
+      <c r="CI1" s="94"/>
+      <c r="CJ1" s="94"/>
+      <c r="CK1" s="94"/>
+      <c r="CL1" s="94"/>
+      <c r="CM1" s="94"/>
+      <c r="CN1" s="94"/>
+      <c r="CO1" s="95"/>
+      <c r="CP1" s="96" t="s">
         <v>2</v>
       </c>
-      <c r="CQ1" s="75"/>
-      <c r="CR1" s="75"/>
-      <c r="CS1" s="75"/>
-      <c r="CT1" s="75"/>
-      <c r="CU1" s="75"/>
-      <c r="CV1" s="75"/>
-      <c r="CW1" s="76"/>
-      <c r="CX1" s="80" t="s">
+      <c r="CQ1" s="97"/>
+      <c r="CR1" s="97"/>
+      <c r="CS1" s="97"/>
+      <c r="CT1" s="97"/>
+      <c r="CU1" s="97"/>
+      <c r="CV1" s="97"/>
+      <c r="CW1" s="98"/>
+      <c r="CX1" s="102" t="s">
         <v>3</v>
       </c>
-      <c r="CY1" s="81"/>
-      <c r="CZ1" s="81"/>
-      <c r="DA1" s="81"/>
-      <c r="DB1" s="81"/>
-      <c r="DC1" s="81"/>
-      <c r="DD1" s="81"/>
-      <c r="DE1" s="81"/>
-      <c r="DF1" s="81"/>
-      <c r="DG1" s="81"/>
-      <c r="DH1" s="81"/>
-      <c r="DI1" s="81"/>
-      <c r="DJ1" s="81"/>
-      <c r="DK1" s="81"/>
-      <c r="DL1" s="81"/>
-      <c r="DM1" s="81"/>
-      <c r="DN1" s="81"/>
-      <c r="DO1" s="81"/>
-      <c r="DP1" s="81"/>
-      <c r="DQ1" s="81"/>
-      <c r="DR1" s="81"/>
-      <c r="DS1" s="81"/>
-      <c r="DT1" s="81"/>
-      <c r="DU1" s="81"/>
-      <c r="DV1" s="81"/>
-      <c r="DW1" s="81"/>
-      <c r="DX1" s="81"/>
-      <c r="DY1" s="81"/>
-      <c r="DZ1" s="81"/>
-      <c r="EA1" s="82"/>
-      <c r="EB1" s="92" t="s">
+      <c r="CY1" s="103"/>
+      <c r="CZ1" s="103"/>
+      <c r="DA1" s="103"/>
+      <c r="DB1" s="103"/>
+      <c r="DC1" s="103"/>
+      <c r="DD1" s="103"/>
+      <c r="DE1" s="103"/>
+      <c r="DF1" s="103"/>
+      <c r="DG1" s="103"/>
+      <c r="DH1" s="103"/>
+      <c r="DI1" s="103"/>
+      <c r="DJ1" s="103"/>
+      <c r="DK1" s="103"/>
+      <c r="DL1" s="103"/>
+      <c r="DM1" s="103"/>
+      <c r="DN1" s="103"/>
+      <c r="DO1" s="103"/>
+      <c r="DP1" s="103"/>
+      <c r="DQ1" s="103"/>
+      <c r="DR1" s="103"/>
+      <c r="DS1" s="103"/>
+      <c r="DT1" s="103"/>
+      <c r="DU1" s="103"/>
+      <c r="DV1" s="103"/>
+      <c r="DW1" s="103"/>
+      <c r="DX1" s="103"/>
+      <c r="DY1" s="103"/>
+      <c r="DZ1" s="103"/>
+      <c r="EA1" s="104"/>
+      <c r="EB1" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="EC1" s="92"/>
-      <c r="ED1" s="92"/>
-      <c r="EE1" s="92"/>
-      <c r="EF1" s="92"/>
-      <c r="EG1" s="92"/>
-      <c r="EH1" s="92"/>
-      <c r="EI1" s="92"/>
-      <c r="EJ1" s="92"/>
-      <c r="EK1" s="92"/>
-      <c r="EL1" s="92"/>
-      <c r="EM1" s="92"/>
-      <c r="EN1" s="92"/>
-      <c r="EO1" s="92"/>
-      <c r="EP1" s="92"/>
+      <c r="EC1" s="73"/>
+      <c r="ED1" s="73"/>
+      <c r="EE1" s="73"/>
+      <c r="EF1" s="73"/>
+      <c r="EG1" s="73"/>
+      <c r="EH1" s="73"/>
+      <c r="EI1" s="73"/>
+      <c r="EJ1" s="73"/>
+      <c r="EK1" s="73"/>
+      <c r="EL1" s="73"/>
+      <c r="EM1" s="73"/>
+      <c r="EN1" s="73"/>
+      <c r="EO1" s="73"/>
+      <c r="EP1" s="73"/>
     </row>
     <row r="2" spans="1:146" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="105" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="105" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="84" t="s">
+      <c r="C2" s="78" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="83" t="s">
+      <c r="D2" s="105" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="64" t="s">
+      <c r="E2" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="64" t="s">
+      <c r="F2" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="64" t="s">
+      <c r="G2" s="68" t="s">
         <v>122</v>
       </c>
-      <c r="H2" s="64" t="s">
+      <c r="H2" s="68" t="s">
         <v>121</v>
       </c>
-      <c r="I2" s="93" t="s">
+      <c r="I2" s="74" t="s">
         <v>110</v>
       </c>
-      <c r="J2" s="94"/>
-      <c r="K2" s="95" t="s">
+      <c r="J2" s="75"/>
+      <c r="K2" s="76" t="s">
         <v>111</v>
       </c>
-      <c r="L2" s="96"/>
-      <c r="M2" s="64" t="s">
+      <c r="L2" s="77"/>
+      <c r="M2" s="68" t="s">
         <v>126</v>
       </c>
-      <c r="N2" s="84" t="s">
+      <c r="N2" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="84" t="s">
+      <c r="O2" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="84" t="s">
+      <c r="P2" s="78" t="s">
         <v>112</v>
       </c>
-      <c r="Q2" s="97" t="s">
+      <c r="Q2" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="97"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="97"/>
-      <c r="U2" s="97"/>
-      <c r="V2" s="97"/>
-      <c r="W2" s="97"/>
-      <c r="X2" s="98" t="s">
+      <c r="R2" s="79"/>
+      <c r="S2" s="79"/>
+      <c r="T2" s="79"/>
+      <c r="U2" s="79"/>
+      <c r="V2" s="79"/>
+      <c r="W2" s="79"/>
+      <c r="X2" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="Y2" s="98"/>
-      <c r="Z2" s="98"/>
-      <c r="AA2" s="98"/>
-      <c r="AB2" s="99" t="s">
+      <c r="Y2" s="80"/>
+      <c r="Z2" s="80"/>
+      <c r="AA2" s="80"/>
+      <c r="AB2" s="81" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="99"/>
-      <c r="AD2" s="99"/>
-      <c r="AE2" s="99"/>
-      <c r="AF2" s="99"/>
-      <c r="AG2" s="99"/>
-      <c r="AH2" s="99"/>
-      <c r="AI2" s="99"/>
-      <c r="AJ2" s="99"/>
-      <c r="AK2" s="100" t="s">
+      <c r="AC2" s="81"/>
+      <c r="AD2" s="81"/>
+      <c r="AE2" s="81"/>
+      <c r="AF2" s="81"/>
+      <c r="AG2" s="81"/>
+      <c r="AH2" s="81"/>
+      <c r="AI2" s="81"/>
+      <c r="AJ2" s="81"/>
+      <c r="AK2" s="82" t="s">
         <v>16</v>
       </c>
-      <c r="AL2" s="100"/>
-      <c r="AM2" s="100"/>
-      <c r="AN2" s="100"/>
-      <c r="AO2" s="100"/>
-      <c r="AP2" s="100"/>
-      <c r="AQ2" s="101" t="s">
+      <c r="AL2" s="82"/>
+      <c r="AM2" s="82"/>
+      <c r="AN2" s="82"/>
+      <c r="AO2" s="82"/>
+      <c r="AP2" s="82"/>
+      <c r="AQ2" s="83" t="s">
         <v>17</v>
       </c>
-      <c r="AR2" s="101"/>
-      <c r="AS2" s="101"/>
-      <c r="AT2" s="101"/>
-      <c r="AU2" s="101"/>
-      <c r="AV2" s="101"/>
-      <c r="AW2" s="101"/>
-      <c r="AX2" s="101"/>
-      <c r="AY2" s="101"/>
-      <c r="AZ2" s="101"/>
-      <c r="BA2" s="101"/>
-      <c r="BB2" s="101"/>
-      <c r="BC2" s="101"/>
-      <c r="BD2" s="101"/>
-      <c r="BE2" s="101"/>
-      <c r="BF2" s="101"/>
-      <c r="BG2" s="101"/>
-      <c r="BH2" s="101"/>
-      <c r="BI2" s="101"/>
-      <c r="BJ2" s="101"/>
-      <c r="BK2" s="101"/>
-      <c r="BL2" s="101"/>
-      <c r="BM2" s="101"/>
-      <c r="BN2" s="102" t="s">
+      <c r="AR2" s="83"/>
+      <c r="AS2" s="83"/>
+      <c r="AT2" s="83"/>
+      <c r="AU2" s="83"/>
+      <c r="AV2" s="83"/>
+      <c r="AW2" s="83"/>
+      <c r="AX2" s="83"/>
+      <c r="AY2" s="83"/>
+      <c r="AZ2" s="83"/>
+      <c r="BA2" s="83"/>
+      <c r="BB2" s="83"/>
+      <c r="BC2" s="83"/>
+      <c r="BD2" s="83"/>
+      <c r="BE2" s="83"/>
+      <c r="BF2" s="83"/>
+      <c r="BG2" s="83"/>
+      <c r="BH2" s="83"/>
+      <c r="BI2" s="83"/>
+      <c r="BJ2" s="83"/>
+      <c r="BK2" s="83"/>
+      <c r="BL2" s="83"/>
+      <c r="BM2" s="83"/>
+      <c r="BN2" s="84" t="s">
         <v>18</v>
       </c>
-      <c r="BO2" s="102"/>
-      <c r="BP2" s="102"/>
-      <c r="BQ2" s="102"/>
-      <c r="BR2" s="102"/>
-      <c r="BS2" s="102"/>
-      <c r="BT2" s="102"/>
-      <c r="BU2" s="102"/>
-      <c r="BV2" s="102"/>
-      <c r="BW2" s="102"/>
-      <c r="BX2" s="102"/>
-      <c r="BY2" s="102"/>
-      <c r="BZ2" s="102"/>
-      <c r="CA2" s="102"/>
-      <c r="CB2" s="102"/>
-      <c r="CC2" s="102"/>
-      <c r="CD2" s="102"/>
-      <c r="CE2" s="102"/>
-      <c r="CF2" s="103" t="s">
+      <c r="BO2" s="84"/>
+      <c r="BP2" s="84"/>
+      <c r="BQ2" s="84"/>
+      <c r="BR2" s="84"/>
+      <c r="BS2" s="84"/>
+      <c r="BT2" s="84"/>
+      <c r="BU2" s="84"/>
+      <c r="BV2" s="84"/>
+      <c r="BW2" s="84"/>
+      <c r="BX2" s="84"/>
+      <c r="BY2" s="84"/>
+      <c r="BZ2" s="84"/>
+      <c r="CA2" s="84"/>
+      <c r="CB2" s="84"/>
+      <c r="CC2" s="84"/>
+      <c r="CD2" s="84"/>
+      <c r="CE2" s="84"/>
+      <c r="CF2" s="85" t="s">
         <v>19</v>
       </c>
-      <c r="CG2" s="103"/>
-      <c r="CH2" s="103"/>
-      <c r="CI2" s="97" t="s">
+      <c r="CG2" s="85"/>
+      <c r="CH2" s="85"/>
+      <c r="CI2" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="CJ2" s="97"/>
-      <c r="CK2" s="97"/>
-      <c r="CL2" s="97"/>
-      <c r="CM2" s="97"/>
-      <c r="CN2" s="97"/>
-      <c r="CO2" s="97"/>
-      <c r="CP2" s="77"/>
-      <c r="CQ2" s="78"/>
-      <c r="CR2" s="78"/>
-      <c r="CS2" s="78"/>
-      <c r="CT2" s="78"/>
-      <c r="CU2" s="78"/>
-      <c r="CV2" s="78"/>
-      <c r="CW2" s="79"/>
-      <c r="CX2" s="104" t="s">
+      <c r="CJ2" s="79"/>
+      <c r="CK2" s="79"/>
+      <c r="CL2" s="79"/>
+      <c r="CM2" s="79"/>
+      <c r="CN2" s="79"/>
+      <c r="CO2" s="79"/>
+      <c r="CP2" s="99"/>
+      <c r="CQ2" s="100"/>
+      <c r="CR2" s="100"/>
+      <c r="CS2" s="100"/>
+      <c r="CT2" s="100"/>
+      <c r="CU2" s="100"/>
+      <c r="CV2" s="100"/>
+      <c r="CW2" s="101"/>
+      <c r="CX2" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="CY2" s="88" t="s">
+      <c r="CY2" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="CZ2" s="89"/>
-      <c r="DA2" s="89"/>
-      <c r="DB2" s="89"/>
-      <c r="DC2" s="89"/>
-      <c r="DD2" s="90"/>
-      <c r="DE2" s="63" t="s">
+      <c r="CZ2" s="70"/>
+      <c r="DA2" s="70"/>
+      <c r="DB2" s="70"/>
+      <c r="DC2" s="70"/>
+      <c r="DD2" s="71"/>
+      <c r="DE2" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="DF2" s="63"/>
-      <c r="DG2" s="63"/>
-      <c r="DH2" s="63"/>
-      <c r="DI2" s="63"/>
-      <c r="DJ2" s="63"/>
-      <c r="DK2" s="63"/>
-      <c r="DL2" s="63"/>
-      <c r="DM2" s="63"/>
-      <c r="DN2" s="63"/>
-      <c r="DO2" s="63"/>
-      <c r="DP2" s="85" t="s">
+      <c r="DF2" s="86"/>
+      <c r="DG2" s="86"/>
+      <c r="DH2" s="86"/>
+      <c r="DI2" s="86"/>
+      <c r="DJ2" s="86"/>
+      <c r="DK2" s="86"/>
+      <c r="DL2" s="86"/>
+      <c r="DM2" s="86"/>
+      <c r="DN2" s="86"/>
+      <c r="DO2" s="86"/>
+      <c r="DP2" s="106" t="s">
         <v>24</v>
       </c>
-      <c r="DQ2" s="86"/>
-      <c r="DR2" s="86"/>
-      <c r="DS2" s="86"/>
-      <c r="DT2" s="86"/>
-      <c r="DU2" s="86"/>
-      <c r="DV2" s="86"/>
-      <c r="DW2" s="86"/>
-      <c r="DX2" s="86"/>
-      <c r="DY2" s="86"/>
-      <c r="DZ2" s="86"/>
-      <c r="EA2" s="87"/>
+      <c r="DQ2" s="107"/>
+      <c r="DR2" s="107"/>
+      <c r="DS2" s="107"/>
+      <c r="DT2" s="107"/>
+      <c r="DU2" s="107"/>
+      <c r="DV2" s="107"/>
+      <c r="DW2" s="107"/>
+      <c r="DX2" s="107"/>
+      <c r="DY2" s="107"/>
+      <c r="DZ2" s="107"/>
+      <c r="EA2" s="108"/>
       <c r="EB2" s="36"/>
       <c r="EC2" s="36"/>
       <c r="ED2" s="36"/>
       <c r="EE2" s="36"/>
-      <c r="EF2" s="106" t="s">
+      <c r="EF2" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="EG2" s="107"/>
-      <c r="EH2" s="107"/>
-      <c r="EI2" s="108"/>
-      <c r="EJ2" s="65" t="s">
+      <c r="EG2" s="66"/>
+      <c r="EH2" s="66"/>
+      <c r="EI2" s="67"/>
+      <c r="EJ2" s="87" t="s">
         <v>26</v>
       </c>
-      <c r="EK2" s="66"/>
-      <c r="EL2" s="66"/>
-      <c r="EM2" s="66"/>
-      <c r="EN2" s="67"/>
-      <c r="EO2" s="91" t="s">
+      <c r="EK2" s="88"/>
+      <c r="EL2" s="88"/>
+      <c r="EM2" s="88"/>
+      <c r="EN2" s="89"/>
+      <c r="EO2" s="72" t="s">
         <v>106</v>
       </c>
-      <c r="EP2" s="91"/>
+      <c r="EP2" s="72"/>
     </row>
     <row r="3" spans="1:146" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="84"/>
-      <c r="B3" s="84"/>
-      <c r="C3" s="84"/>
-      <c r="D3" s="84"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
+      <c r="A3" s="78"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
       <c r="I3" s="34" t="s">
         <v>8</v>
       </c>
@@ -2632,10 +2629,10 @@
       <c r="L3" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="64"/>
-      <c r="N3" s="84"/>
-      <c r="O3" s="84"/>
-      <c r="P3" s="84"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="78"/>
+      <c r="O3" s="78"/>
+      <c r="P3" s="78"/>
       <c r="Q3" s="37" t="s">
         <v>27</v>
       </c>
@@ -2891,7 +2888,7 @@
       <c r="CW3" s="52" t="s">
         <v>70</v>
       </c>
-      <c r="CX3" s="105"/>
+      <c r="CX3" s="64"/>
       <c r="CY3" s="53" t="s">
         <v>71</v>
       </c>
@@ -3026,20 +3023,17 @@
       </c>
     </row>
     <row r="4" spans="1:146" x14ac:dyDescent="0.25">
-      <c r="O4" s="33" t="s">
-        <v>269</v>
-      </c>
-      <c r="P4" s="33" cm="1">
+      <c r="P4" s="33" t="str" cm="1">
         <f t="array" ref="P4">IFERROR(SUM(VALUE(_xlfn.TEXTSPLIT(O4, ";"))), "")</f>
-        <v>5</v>
+        <v/>
       </c>
       <c r="DO4" t="str">
         <f>IF(SUM(DE4:DN4)=0, "", SUM(DE4:DN4))</f>
         <v/>
       </c>
-      <c r="EP4">
+      <c r="EP4" t="str">
         <f>IFERROR(P4-EO4, "")</f>
-        <v>5</v>
+        <v/>
       </c>
     </row>
     <row r="5" spans="1:146" x14ac:dyDescent="0.25">
@@ -33206,11 +33200,18 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="CX2:CX3"/>
-    <mergeCell ref="EF2:EI2"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="CY2:DD2"/>
-    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="Q1:CO1"/>
+    <mergeCell ref="CP1:CW2"/>
+    <mergeCell ref="CX1:EA1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="DP2:EA2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
     <mergeCell ref="EO2:EP2"/>
     <mergeCell ref="EB1:EP1"/>
     <mergeCell ref="I2:J2"/>
@@ -33225,21 +33226,14 @@
     <mergeCell ref="CF2:CH2"/>
     <mergeCell ref="CI2:CO2"/>
     <mergeCell ref="DE2:DO2"/>
-    <mergeCell ref="G2:G3"/>
     <mergeCell ref="EJ2:EN2"/>
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="Q1:CO1"/>
-    <mergeCell ref="CP1:CW2"/>
-    <mergeCell ref="CX1:EA1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="DP2:EA2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="CX2:CX3"/>
+    <mergeCell ref="EF2:EI2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="CY2:DD2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <dataValidations xWindow="509" yWindow="477" count="6">
     <dataValidation type="list" allowBlank="1" sqref="A3" xr:uid="{C94C9C08-E811-49C1-A6EE-6ABF7BB7DF7D}">
@@ -33324,378 +33318,378 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:146" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="134" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="110"/>
-      <c r="C1" s="110"/>
-      <c r="D1" s="110"/>
-      <c r="E1" s="110"/>
-      <c r="F1" s="110"/>
-      <c r="G1" s="110"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="110"/>
-      <c r="K1" s="110"/>
-      <c r="L1" s="110"/>
-      <c r="M1" s="110"/>
-      <c r="N1" s="110"/>
-      <c r="O1" s="110"/>
-      <c r="P1" s="111"/>
-      <c r="Q1" s="112" t="s">
+      <c r="B1" s="135"/>
+      <c r="C1" s="135"/>
+      <c r="D1" s="135"/>
+      <c r="E1" s="135"/>
+      <c r="F1" s="135"/>
+      <c r="G1" s="135"/>
+      <c r="H1" s="135"/>
+      <c r="I1" s="135"/>
+      <c r="J1" s="135"/>
+      <c r="K1" s="135"/>
+      <c r="L1" s="135"/>
+      <c r="M1" s="135"/>
+      <c r="N1" s="135"/>
+      <c r="O1" s="135"/>
+      <c r="P1" s="136"/>
+      <c r="Q1" s="137" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="113"/>
-      <c r="S1" s="113"/>
-      <c r="T1" s="113"/>
-      <c r="U1" s="113"/>
-      <c r="V1" s="113"/>
-      <c r="W1" s="113"/>
-      <c r="X1" s="113"/>
-      <c r="Y1" s="113"/>
-      <c r="Z1" s="113"/>
-      <c r="AA1" s="113"/>
-      <c r="AB1" s="113"/>
-      <c r="AC1" s="113"/>
-      <c r="AD1" s="113"/>
-      <c r="AE1" s="113"/>
-      <c r="AF1" s="113"/>
-      <c r="AG1" s="113"/>
-      <c r="AH1" s="113"/>
-      <c r="AI1" s="113"/>
-      <c r="AJ1" s="113"/>
-      <c r="AK1" s="113"/>
-      <c r="AL1" s="113"/>
-      <c r="AM1" s="113"/>
-      <c r="AN1" s="113"/>
-      <c r="AO1" s="113"/>
-      <c r="AP1" s="113"/>
-      <c r="AQ1" s="113"/>
-      <c r="AR1" s="113"/>
-      <c r="AS1" s="113"/>
-      <c r="AT1" s="113"/>
-      <c r="AU1" s="113"/>
-      <c r="AV1" s="113"/>
-      <c r="AW1" s="113"/>
-      <c r="AX1" s="113"/>
-      <c r="AY1" s="113"/>
-      <c r="AZ1" s="113"/>
-      <c r="BA1" s="113"/>
-      <c r="BB1" s="113"/>
-      <c r="BC1" s="113"/>
-      <c r="BD1" s="113"/>
-      <c r="BE1" s="113"/>
-      <c r="BF1" s="113"/>
-      <c r="BG1" s="113"/>
-      <c r="BH1" s="113"/>
-      <c r="BI1" s="113"/>
-      <c r="BJ1" s="113"/>
-      <c r="BK1" s="113"/>
-      <c r="BL1" s="113"/>
-      <c r="BM1" s="113"/>
-      <c r="BN1" s="113"/>
-      <c r="BO1" s="113"/>
-      <c r="BP1" s="113"/>
-      <c r="BQ1" s="113"/>
-      <c r="BR1" s="113"/>
-      <c r="BS1" s="113"/>
-      <c r="BT1" s="113"/>
-      <c r="BU1" s="113"/>
-      <c r="BV1" s="113"/>
-      <c r="BW1" s="113"/>
-      <c r="BX1" s="113"/>
-      <c r="BY1" s="113"/>
-      <c r="BZ1" s="113"/>
-      <c r="CA1" s="113"/>
-      <c r="CB1" s="113"/>
-      <c r="CC1" s="113"/>
-      <c r="CD1" s="113"/>
-      <c r="CE1" s="113"/>
-      <c r="CF1" s="113"/>
-      <c r="CG1" s="113"/>
-      <c r="CH1" s="113"/>
-      <c r="CI1" s="113"/>
-      <c r="CJ1" s="113"/>
-      <c r="CK1" s="113"/>
-      <c r="CL1" s="113"/>
-      <c r="CM1" s="113"/>
-      <c r="CN1" s="113"/>
-      <c r="CO1" s="114"/>
-      <c r="CP1" s="115" t="s">
+      <c r="R1" s="138"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="138"/>
+      <c r="U1" s="138"/>
+      <c r="V1" s="138"/>
+      <c r="W1" s="138"/>
+      <c r="X1" s="138"/>
+      <c r="Y1" s="138"/>
+      <c r="Z1" s="138"/>
+      <c r="AA1" s="138"/>
+      <c r="AB1" s="138"/>
+      <c r="AC1" s="138"/>
+      <c r="AD1" s="138"/>
+      <c r="AE1" s="138"/>
+      <c r="AF1" s="138"/>
+      <c r="AG1" s="138"/>
+      <c r="AH1" s="138"/>
+      <c r="AI1" s="138"/>
+      <c r="AJ1" s="138"/>
+      <c r="AK1" s="138"/>
+      <c r="AL1" s="138"/>
+      <c r="AM1" s="138"/>
+      <c r="AN1" s="138"/>
+      <c r="AO1" s="138"/>
+      <c r="AP1" s="138"/>
+      <c r="AQ1" s="138"/>
+      <c r="AR1" s="138"/>
+      <c r="AS1" s="138"/>
+      <c r="AT1" s="138"/>
+      <c r="AU1" s="138"/>
+      <c r="AV1" s="138"/>
+      <c r="AW1" s="138"/>
+      <c r="AX1" s="138"/>
+      <c r="AY1" s="138"/>
+      <c r="AZ1" s="138"/>
+      <c r="BA1" s="138"/>
+      <c r="BB1" s="138"/>
+      <c r="BC1" s="138"/>
+      <c r="BD1" s="138"/>
+      <c r="BE1" s="138"/>
+      <c r="BF1" s="138"/>
+      <c r="BG1" s="138"/>
+      <c r="BH1" s="138"/>
+      <c r="BI1" s="138"/>
+      <c r="BJ1" s="138"/>
+      <c r="BK1" s="138"/>
+      <c r="BL1" s="138"/>
+      <c r="BM1" s="138"/>
+      <c r="BN1" s="138"/>
+      <c r="BO1" s="138"/>
+      <c r="BP1" s="138"/>
+      <c r="BQ1" s="138"/>
+      <c r="BR1" s="138"/>
+      <c r="BS1" s="138"/>
+      <c r="BT1" s="138"/>
+      <c r="BU1" s="138"/>
+      <c r="BV1" s="138"/>
+      <c r="BW1" s="138"/>
+      <c r="BX1" s="138"/>
+      <c r="BY1" s="138"/>
+      <c r="BZ1" s="138"/>
+      <c r="CA1" s="138"/>
+      <c r="CB1" s="138"/>
+      <c r="CC1" s="138"/>
+      <c r="CD1" s="138"/>
+      <c r="CE1" s="138"/>
+      <c r="CF1" s="138"/>
+      <c r="CG1" s="138"/>
+      <c r="CH1" s="138"/>
+      <c r="CI1" s="138"/>
+      <c r="CJ1" s="138"/>
+      <c r="CK1" s="138"/>
+      <c r="CL1" s="138"/>
+      <c r="CM1" s="138"/>
+      <c r="CN1" s="138"/>
+      <c r="CO1" s="139"/>
+      <c r="CP1" s="140" t="s">
         <v>2</v>
       </c>
-      <c r="CQ1" s="116"/>
-      <c r="CR1" s="116"/>
-      <c r="CS1" s="116"/>
-      <c r="CT1" s="116"/>
-      <c r="CU1" s="116"/>
-      <c r="CV1" s="116"/>
-      <c r="CW1" s="117"/>
-      <c r="CX1" s="121" t="s">
+      <c r="CQ1" s="141"/>
+      <c r="CR1" s="141"/>
+      <c r="CS1" s="141"/>
+      <c r="CT1" s="141"/>
+      <c r="CU1" s="141"/>
+      <c r="CV1" s="141"/>
+      <c r="CW1" s="142"/>
+      <c r="CX1" s="146" t="s">
         <v>3</v>
       </c>
-      <c r="CY1" s="122"/>
-      <c r="CZ1" s="122"/>
-      <c r="DA1" s="122"/>
-      <c r="DB1" s="122"/>
-      <c r="DC1" s="122"/>
-      <c r="DD1" s="122"/>
-      <c r="DE1" s="122"/>
-      <c r="DF1" s="122"/>
-      <c r="DG1" s="122"/>
-      <c r="DH1" s="122"/>
-      <c r="DI1" s="122"/>
-      <c r="DJ1" s="122"/>
-      <c r="DK1" s="122"/>
-      <c r="DL1" s="122"/>
-      <c r="DM1" s="122"/>
-      <c r="DN1" s="122"/>
-      <c r="DO1" s="122"/>
-      <c r="DP1" s="122"/>
-      <c r="DQ1" s="122"/>
-      <c r="DR1" s="122"/>
-      <c r="DS1" s="122"/>
-      <c r="DT1" s="122"/>
-      <c r="DU1" s="122"/>
-      <c r="DV1" s="122"/>
-      <c r="DW1" s="122"/>
-      <c r="DX1" s="122"/>
-      <c r="DY1" s="122"/>
-      <c r="DZ1" s="122"/>
-      <c r="EA1" s="123"/>
-      <c r="EB1" s="124" t="s">
+      <c r="CY1" s="147"/>
+      <c r="CZ1" s="147"/>
+      <c r="DA1" s="147"/>
+      <c r="DB1" s="147"/>
+      <c r="DC1" s="147"/>
+      <c r="DD1" s="147"/>
+      <c r="DE1" s="147"/>
+      <c r="DF1" s="147"/>
+      <c r="DG1" s="147"/>
+      <c r="DH1" s="147"/>
+      <c r="DI1" s="147"/>
+      <c r="DJ1" s="147"/>
+      <c r="DK1" s="147"/>
+      <c r="DL1" s="147"/>
+      <c r="DM1" s="147"/>
+      <c r="DN1" s="147"/>
+      <c r="DO1" s="147"/>
+      <c r="DP1" s="147"/>
+      <c r="DQ1" s="147"/>
+      <c r="DR1" s="147"/>
+      <c r="DS1" s="147"/>
+      <c r="DT1" s="147"/>
+      <c r="DU1" s="147"/>
+      <c r="DV1" s="147"/>
+      <c r="DW1" s="147"/>
+      <c r="DX1" s="147"/>
+      <c r="DY1" s="147"/>
+      <c r="DZ1" s="147"/>
+      <c r="EA1" s="148"/>
+      <c r="EB1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="EC1" s="124"/>
-      <c r="ED1" s="124"/>
-      <c r="EE1" s="124"/>
-      <c r="EF1" s="124"/>
-      <c r="EG1" s="124"/>
-      <c r="EH1" s="124"/>
-      <c r="EI1" s="124"/>
-      <c r="EJ1" s="124"/>
-      <c r="EK1" s="124"/>
-      <c r="EL1" s="124"/>
-      <c r="EM1" s="124"/>
-      <c r="EN1" s="124"/>
-      <c r="EO1" s="124"/>
-      <c r="EP1" s="124"/>
+      <c r="EC1" s="149"/>
+      <c r="ED1" s="149"/>
+      <c r="EE1" s="149"/>
+      <c r="EF1" s="149"/>
+      <c r="EG1" s="149"/>
+      <c r="EH1" s="149"/>
+      <c r="EI1" s="149"/>
+      <c r="EJ1" s="149"/>
+      <c r="EK1" s="149"/>
+      <c r="EL1" s="149"/>
+      <c r="EM1" s="149"/>
+      <c r="EN1" s="149"/>
+      <c r="EO1" s="149"/>
+      <c r="EP1" s="149"/>
     </row>
     <row r="2" spans="1:146" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="125" t="s">
+      <c r="A2" s="150" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="150" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="127" t="s">
+      <c r="C2" s="132" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="125" t="s">
+      <c r="D2" s="150" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="128" t="s">
+      <c r="E2" s="130" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="128" t="s">
+      <c r="F2" s="130" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="128" t="s">
+      <c r="G2" s="130" t="s">
         <v>122</v>
       </c>
-      <c r="H2" s="128" t="s">
+      <c r="H2" s="130" t="s">
         <v>121</v>
       </c>
-      <c r="I2" s="131" t="s">
+      <c r="I2" s="152" t="s">
         <v>110</v>
       </c>
-      <c r="J2" s="132"/>
-      <c r="K2" s="133" t="s">
+      <c r="J2" s="153"/>
+      <c r="K2" s="154" t="s">
         <v>111</v>
       </c>
-      <c r="L2" s="134"/>
-      <c r="M2" s="128" t="s">
+      <c r="L2" s="155"/>
+      <c r="M2" s="130" t="s">
         <v>126</v>
       </c>
-      <c r="N2" s="127" t="s">
+      <c r="N2" s="132" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="127" t="s">
+      <c r="O2" s="132" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="127" t="s">
+      <c r="P2" s="132" t="s">
         <v>112</v>
       </c>
-      <c r="Q2" s="135" t="s">
+      <c r="Q2" s="115" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="135"/>
-      <c r="S2" s="135"/>
-      <c r="T2" s="135"/>
-      <c r="U2" s="135"/>
-      <c r="V2" s="135"/>
-      <c r="W2" s="135"/>
-      <c r="X2" s="136" t="s">
+      <c r="R2" s="115"/>
+      <c r="S2" s="115"/>
+      <c r="T2" s="115"/>
+      <c r="U2" s="115"/>
+      <c r="V2" s="115"/>
+      <c r="W2" s="115"/>
+      <c r="X2" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="Y2" s="136"/>
-      <c r="Z2" s="136"/>
-      <c r="AA2" s="136"/>
-      <c r="AB2" s="130" t="s">
+      <c r="Y2" s="109"/>
+      <c r="Z2" s="109"/>
+      <c r="AA2" s="109"/>
+      <c r="AB2" s="151" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="130"/>
-      <c r="AD2" s="130"/>
-      <c r="AE2" s="130"/>
-      <c r="AF2" s="130"/>
-      <c r="AG2" s="130"/>
-      <c r="AH2" s="130"/>
-      <c r="AI2" s="130"/>
-      <c r="AJ2" s="130"/>
-      <c r="AK2" s="138" t="s">
+      <c r="AC2" s="151"/>
+      <c r="AD2" s="151"/>
+      <c r="AE2" s="151"/>
+      <c r="AF2" s="151"/>
+      <c r="AG2" s="151"/>
+      <c r="AH2" s="151"/>
+      <c r="AI2" s="151"/>
+      <c r="AJ2" s="151"/>
+      <c r="AK2" s="111" t="s">
         <v>16</v>
       </c>
-      <c r="AL2" s="138"/>
-      <c r="AM2" s="138"/>
-      <c r="AN2" s="138"/>
-      <c r="AO2" s="138"/>
-      <c r="AP2" s="138"/>
-      <c r="AQ2" s="139" t="s">
+      <c r="AL2" s="111"/>
+      <c r="AM2" s="111"/>
+      <c r="AN2" s="111"/>
+      <c r="AO2" s="111"/>
+      <c r="AP2" s="111"/>
+      <c r="AQ2" s="112" t="s">
         <v>17</v>
       </c>
-      <c r="AR2" s="139"/>
-      <c r="AS2" s="139"/>
-      <c r="AT2" s="139"/>
-      <c r="AU2" s="139"/>
-      <c r="AV2" s="139"/>
-      <c r="AW2" s="139"/>
-      <c r="AX2" s="139"/>
-      <c r="AY2" s="139"/>
-      <c r="AZ2" s="139"/>
-      <c r="BA2" s="139"/>
-      <c r="BB2" s="139"/>
-      <c r="BC2" s="139"/>
-      <c r="BD2" s="139"/>
-      <c r="BE2" s="139"/>
-      <c r="BF2" s="139"/>
-      <c r="BG2" s="139"/>
-      <c r="BH2" s="139"/>
-      <c r="BI2" s="139"/>
-      <c r="BJ2" s="139"/>
-      <c r="BK2" s="139"/>
-      <c r="BL2" s="139"/>
-      <c r="BM2" s="139"/>
-      <c r="BN2" s="140" t="s">
+      <c r="AR2" s="112"/>
+      <c r="AS2" s="112"/>
+      <c r="AT2" s="112"/>
+      <c r="AU2" s="112"/>
+      <c r="AV2" s="112"/>
+      <c r="AW2" s="112"/>
+      <c r="AX2" s="112"/>
+      <c r="AY2" s="112"/>
+      <c r="AZ2" s="112"/>
+      <c r="BA2" s="112"/>
+      <c r="BB2" s="112"/>
+      <c r="BC2" s="112"/>
+      <c r="BD2" s="112"/>
+      <c r="BE2" s="112"/>
+      <c r="BF2" s="112"/>
+      <c r="BG2" s="112"/>
+      <c r="BH2" s="112"/>
+      <c r="BI2" s="112"/>
+      <c r="BJ2" s="112"/>
+      <c r="BK2" s="112"/>
+      <c r="BL2" s="112"/>
+      <c r="BM2" s="112"/>
+      <c r="BN2" s="113" t="s">
         <v>18</v>
       </c>
-      <c r="BO2" s="140"/>
-      <c r="BP2" s="140"/>
-      <c r="BQ2" s="140"/>
-      <c r="BR2" s="140"/>
-      <c r="BS2" s="140"/>
-      <c r="BT2" s="140"/>
-      <c r="BU2" s="140"/>
-      <c r="BV2" s="140"/>
-      <c r="BW2" s="140"/>
-      <c r="BX2" s="140"/>
-      <c r="BY2" s="140"/>
-      <c r="BZ2" s="140"/>
-      <c r="CA2" s="140"/>
-      <c r="CB2" s="140"/>
-      <c r="CC2" s="140"/>
-      <c r="CD2" s="140"/>
-      <c r="CE2" s="140"/>
-      <c r="CF2" s="141" t="s">
+      <c r="BO2" s="113"/>
+      <c r="BP2" s="113"/>
+      <c r="BQ2" s="113"/>
+      <c r="BR2" s="113"/>
+      <c r="BS2" s="113"/>
+      <c r="BT2" s="113"/>
+      <c r="BU2" s="113"/>
+      <c r="BV2" s="113"/>
+      <c r="BW2" s="113"/>
+      <c r="BX2" s="113"/>
+      <c r="BY2" s="113"/>
+      <c r="BZ2" s="113"/>
+      <c r="CA2" s="113"/>
+      <c r="CB2" s="113"/>
+      <c r="CC2" s="113"/>
+      <c r="CD2" s="113"/>
+      <c r="CE2" s="113"/>
+      <c r="CF2" s="114" t="s">
         <v>19</v>
       </c>
-      <c r="CG2" s="141"/>
-      <c r="CH2" s="141"/>
-      <c r="CI2" s="135" t="s">
+      <c r="CG2" s="114"/>
+      <c r="CH2" s="114"/>
+      <c r="CI2" s="115" t="s">
         <v>20</v>
       </c>
-      <c r="CJ2" s="135"/>
-      <c r="CK2" s="135"/>
-      <c r="CL2" s="135"/>
-      <c r="CM2" s="135"/>
-      <c r="CN2" s="135"/>
-      <c r="CO2" s="135"/>
-      <c r="CP2" s="118"/>
-      <c r="CQ2" s="119"/>
-      <c r="CR2" s="119"/>
-      <c r="CS2" s="119"/>
-      <c r="CT2" s="119"/>
-      <c r="CU2" s="119"/>
-      <c r="CV2" s="119"/>
-      <c r="CW2" s="120"/>
-      <c r="CX2" s="142" t="s">
+      <c r="CJ2" s="115"/>
+      <c r="CK2" s="115"/>
+      <c r="CL2" s="115"/>
+      <c r="CM2" s="115"/>
+      <c r="CN2" s="115"/>
+      <c r="CO2" s="115"/>
+      <c r="CP2" s="143"/>
+      <c r="CQ2" s="144"/>
+      <c r="CR2" s="144"/>
+      <c r="CS2" s="144"/>
+      <c r="CT2" s="144"/>
+      <c r="CU2" s="144"/>
+      <c r="CV2" s="144"/>
+      <c r="CW2" s="145"/>
+      <c r="CX2" s="116" t="s">
         <v>21</v>
       </c>
-      <c r="CY2" s="144" t="s">
+      <c r="CY2" s="118" t="s">
         <v>22</v>
       </c>
-      <c r="CZ2" s="145"/>
-      <c r="DA2" s="145"/>
-      <c r="DB2" s="145"/>
-      <c r="DC2" s="145"/>
-      <c r="DD2" s="146"/>
-      <c r="DE2" s="63" t="s">
+      <c r="CZ2" s="119"/>
+      <c r="DA2" s="119"/>
+      <c r="DB2" s="119"/>
+      <c r="DC2" s="119"/>
+      <c r="DD2" s="120"/>
+      <c r="DE2" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="DF2" s="63"/>
-      <c r="DG2" s="63"/>
-      <c r="DH2" s="63"/>
-      <c r="DI2" s="63"/>
-      <c r="DJ2" s="63"/>
-      <c r="DK2" s="63"/>
-      <c r="DL2" s="63"/>
-      <c r="DM2" s="63"/>
-      <c r="DN2" s="63"/>
-      <c r="DO2" s="63"/>
-      <c r="DP2" s="147" t="s">
+      <c r="DF2" s="86"/>
+      <c r="DG2" s="86"/>
+      <c r="DH2" s="86"/>
+      <c r="DI2" s="86"/>
+      <c r="DJ2" s="86"/>
+      <c r="DK2" s="86"/>
+      <c r="DL2" s="86"/>
+      <c r="DM2" s="86"/>
+      <c r="DN2" s="86"/>
+      <c r="DO2" s="86"/>
+      <c r="DP2" s="121" t="s">
         <v>24</v>
       </c>
-      <c r="DQ2" s="148"/>
-      <c r="DR2" s="148"/>
-      <c r="DS2" s="148"/>
-      <c r="DT2" s="148"/>
-      <c r="DU2" s="148"/>
-      <c r="DV2" s="148"/>
-      <c r="DW2" s="148"/>
-      <c r="DX2" s="148"/>
-      <c r="DY2" s="148"/>
-      <c r="DZ2" s="148"/>
-      <c r="EA2" s="149"/>
+      <c r="DQ2" s="122"/>
+      <c r="DR2" s="122"/>
+      <c r="DS2" s="122"/>
+      <c r="DT2" s="122"/>
+      <c r="DU2" s="122"/>
+      <c r="DV2" s="122"/>
+      <c r="DW2" s="122"/>
+      <c r="DX2" s="122"/>
+      <c r="DY2" s="122"/>
+      <c r="DZ2" s="122"/>
+      <c r="EA2" s="123"/>
       <c r="EB2" s="1"/>
       <c r="EC2" s="1"/>
       <c r="ED2" s="1"/>
       <c r="EE2" s="1"/>
-      <c r="EF2" s="150" t="s">
+      <c r="EF2" s="124" t="s">
         <v>25</v>
       </c>
-      <c r="EG2" s="151"/>
-      <c r="EH2" s="151"/>
-      <c r="EI2" s="152"/>
-      <c r="EJ2" s="153" t="s">
+      <c r="EG2" s="125"/>
+      <c r="EH2" s="125"/>
+      <c r="EI2" s="126"/>
+      <c r="EJ2" s="127" t="s">
         <v>26</v>
       </c>
-      <c r="EK2" s="154"/>
-      <c r="EL2" s="154"/>
-      <c r="EM2" s="154"/>
-      <c r="EN2" s="155"/>
-      <c r="EO2" s="137" t="s">
+      <c r="EK2" s="128"/>
+      <c r="EL2" s="128"/>
+      <c r="EM2" s="128"/>
+      <c r="EN2" s="129"/>
+      <c r="EO2" s="110" t="s">
         <v>106</v>
       </c>
-      <c r="EP2" s="137"/>
+      <c r="EP2" s="110"/>
     </row>
     <row r="3" spans="1:146" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="126"/>
-      <c r="B3" s="126"/>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="129"/>
-      <c r="F3" s="129"/>
-      <c r="G3" s="129"/>
-      <c r="H3" s="129"/>
+      <c r="A3" s="133"/>
+      <c r="B3" s="133"/>
+      <c r="C3" s="133"/>
+      <c r="D3" s="133"/>
+      <c r="E3" s="131"/>
+      <c r="F3" s="131"/>
+      <c r="G3" s="131"/>
+      <c r="H3" s="131"/>
       <c r="I3" s="2" t="s">
         <v>8</v>
       </c>
@@ -33708,10 +33702,10 @@
       <c r="L3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="129"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="126"/>
+      <c r="M3" s="131"/>
+      <c r="N3" s="133"/>
+      <c r="O3" s="133"/>
+      <c r="P3" s="133"/>
       <c r="Q3" s="4" t="s">
         <v>27</v>
       </c>
@@ -33967,7 +33961,7 @@
       <c r="CW3" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="CX3" s="143"/>
+      <c r="CX3" s="117"/>
       <c r="CY3" s="21" t="s">
         <v>71</v>
       </c>
@@ -34608,24 +34602,6 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="X2:AA2"/>
-    <mergeCell ref="EO2:EP2"/>
-    <mergeCell ref="AK2:AP2"/>
-    <mergeCell ref="AQ2:BM2"/>
-    <mergeCell ref="BN2:CE2"/>
-    <mergeCell ref="CF2:CH2"/>
-    <mergeCell ref="CI2:CO2"/>
-    <mergeCell ref="CX2:CX3"/>
-    <mergeCell ref="CY2:DD2"/>
-    <mergeCell ref="DE2:DO2"/>
-    <mergeCell ref="DP2:EA2"/>
-    <mergeCell ref="EF2:EI2"/>
-    <mergeCell ref="EJ2:EN2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:W2"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="Q1:CO1"/>
     <mergeCell ref="CP1:CW2"/>
@@ -34642,6 +34618,24 @@
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:W2"/>
+    <mergeCell ref="X2:AA2"/>
+    <mergeCell ref="EO2:EP2"/>
+    <mergeCell ref="AK2:AP2"/>
+    <mergeCell ref="AQ2:BM2"/>
+    <mergeCell ref="BN2:CE2"/>
+    <mergeCell ref="CF2:CH2"/>
+    <mergeCell ref="CI2:CO2"/>
+    <mergeCell ref="CX2:CX3"/>
+    <mergeCell ref="CY2:DD2"/>
+    <mergeCell ref="DE2:DO2"/>
+    <mergeCell ref="DP2:EA2"/>
+    <mergeCell ref="EF2:EI2"/>
+    <mergeCell ref="EJ2:EN2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="B3" xr:uid="{ACD79C73-1AC5-4E5C-B174-8735C17FE353}">

</xml_diff>

<commit_message>
Update API process new
</commit_message>
<xml_diff>
--- a/src/main/resources/static/Sample_Excel_Import_Asset.xlsx
+++ b/src/main/resources/static/Sample_Excel_Import_Asset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CompanyBk\CSVC\csvc-hust\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE37ABA2-FAA3-411C-9B65-91C275001F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28976C95-FE9A-4EC6-901A-E9D8B05CF3F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{71050258-D013-4370-AEE7-AC2797CFA723}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="258">
   <si>
     <t>Thông tin chung</t>
   </si>
@@ -992,6 +992,9 @@
   <si>
     <t>Danh sách các nguồn hình thành:</t>
   </si>
+  <si>
+    <t>Vật kiến trúc</t>
+  </si>
 </sst>
 </file>
 
@@ -1571,25 +1574,64 @@
     <xf numFmtId="0" fontId="3" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="19" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="19" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="15" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1608,9 +1650,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1655,133 +1694,22 @@
     <xf numFmtId="49" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="19" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="15" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="19" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1835,6 +1763,18 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1848,6 +1788,69 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2211,197 +2214,197 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:146" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="100" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
-      <c r="N1" s="89"/>
-      <c r="O1" s="89"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="91" t="s">
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="101"/>
+      <c r="H1" s="101"/>
+      <c r="I1" s="101"/>
+      <c r="J1" s="101"/>
+      <c r="K1" s="101"/>
+      <c r="L1" s="101"/>
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="102"/>
+      <c r="Q1" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="92"/>
-      <c r="S1" s="92"/>
-      <c r="T1" s="92"/>
-      <c r="U1" s="92"/>
-      <c r="V1" s="92"/>
-      <c r="W1" s="92"/>
-      <c r="X1" s="92"/>
-      <c r="Y1" s="92"/>
-      <c r="Z1" s="92"/>
-      <c r="AA1" s="92"/>
-      <c r="AB1" s="92"/>
-      <c r="AC1" s="92"/>
-      <c r="AD1" s="92"/>
-      <c r="AE1" s="92"/>
-      <c r="AF1" s="92"/>
-      <c r="AG1" s="92"/>
-      <c r="AH1" s="92"/>
-      <c r="AI1" s="92"/>
-      <c r="AJ1" s="92"/>
-      <c r="AK1" s="92"/>
-      <c r="AL1" s="92"/>
-      <c r="AM1" s="92"/>
-      <c r="AN1" s="92"/>
-      <c r="AO1" s="92"/>
-      <c r="AP1" s="92"/>
-      <c r="AQ1" s="92"/>
-      <c r="AR1" s="92"/>
-      <c r="AS1" s="92"/>
-      <c r="AT1" s="92"/>
-      <c r="AU1" s="92"/>
-      <c r="AV1" s="92"/>
-      <c r="AW1" s="92"/>
-      <c r="AX1" s="92"/>
-      <c r="AY1" s="92"/>
-      <c r="AZ1" s="92"/>
-      <c r="BA1" s="92"/>
-      <c r="BB1" s="92"/>
-      <c r="BC1" s="92"/>
-      <c r="BD1" s="92"/>
-      <c r="BE1" s="92"/>
-      <c r="BF1" s="92"/>
-      <c r="BG1" s="92"/>
-      <c r="BH1" s="92"/>
-      <c r="BI1" s="92"/>
-      <c r="BJ1" s="92"/>
-      <c r="BK1" s="92"/>
-      <c r="BL1" s="92"/>
-      <c r="BM1" s="92"/>
-      <c r="BN1" s="92"/>
-      <c r="BO1" s="92"/>
-      <c r="BP1" s="92"/>
-      <c r="BQ1" s="92"/>
-      <c r="BR1" s="92"/>
-      <c r="BS1" s="92"/>
-      <c r="BT1" s="92"/>
-      <c r="BU1" s="92"/>
-      <c r="BV1" s="92"/>
-      <c r="BW1" s="92"/>
-      <c r="BX1" s="92"/>
-      <c r="BY1" s="92"/>
-      <c r="BZ1" s="92"/>
-      <c r="CA1" s="92"/>
-      <c r="CB1" s="92"/>
-      <c r="CC1" s="92"/>
-      <c r="CD1" s="92"/>
-      <c r="CE1" s="92"/>
-      <c r="CF1" s="92"/>
-      <c r="CG1" s="92"/>
-      <c r="CH1" s="92"/>
-      <c r="CI1" s="92"/>
-      <c r="CJ1" s="92"/>
-      <c r="CK1" s="92"/>
-      <c r="CL1" s="92"/>
-      <c r="CM1" s="92"/>
-      <c r="CN1" s="92"/>
-      <c r="CO1" s="93"/>
-      <c r="CP1" s="94" t="s">
+      <c r="R1" s="64"/>
+      <c r="S1" s="64"/>
+      <c r="T1" s="64"/>
+      <c r="U1" s="64"/>
+      <c r="V1" s="64"/>
+      <c r="W1" s="64"/>
+      <c r="X1" s="64"/>
+      <c r="Y1" s="64"/>
+      <c r="Z1" s="64"/>
+      <c r="AA1" s="64"/>
+      <c r="AB1" s="64"/>
+      <c r="AC1" s="64"/>
+      <c r="AD1" s="64"/>
+      <c r="AE1" s="64"/>
+      <c r="AF1" s="64"/>
+      <c r="AG1" s="64"/>
+      <c r="AH1" s="64"/>
+      <c r="AI1" s="64"/>
+      <c r="AJ1" s="64"/>
+      <c r="AK1" s="64"/>
+      <c r="AL1" s="64"/>
+      <c r="AM1" s="64"/>
+      <c r="AN1" s="64"/>
+      <c r="AO1" s="64"/>
+      <c r="AP1" s="64"/>
+      <c r="AQ1" s="64"/>
+      <c r="AR1" s="64"/>
+      <c r="AS1" s="64"/>
+      <c r="AT1" s="64"/>
+      <c r="AU1" s="64"/>
+      <c r="AV1" s="64"/>
+      <c r="AW1" s="64"/>
+      <c r="AX1" s="64"/>
+      <c r="AY1" s="64"/>
+      <c r="AZ1" s="64"/>
+      <c r="BA1" s="64"/>
+      <c r="BB1" s="64"/>
+      <c r="BC1" s="64"/>
+      <c r="BD1" s="64"/>
+      <c r="BE1" s="64"/>
+      <c r="BF1" s="64"/>
+      <c r="BG1" s="64"/>
+      <c r="BH1" s="64"/>
+      <c r="BI1" s="64"/>
+      <c r="BJ1" s="64"/>
+      <c r="BK1" s="64"/>
+      <c r="BL1" s="64"/>
+      <c r="BM1" s="64"/>
+      <c r="BN1" s="64"/>
+      <c r="BO1" s="64"/>
+      <c r="BP1" s="64"/>
+      <c r="BQ1" s="64"/>
+      <c r="BR1" s="64"/>
+      <c r="BS1" s="64"/>
+      <c r="BT1" s="64"/>
+      <c r="BU1" s="64"/>
+      <c r="BV1" s="64"/>
+      <c r="BW1" s="64"/>
+      <c r="BX1" s="64"/>
+      <c r="BY1" s="64"/>
+      <c r="BZ1" s="64"/>
+      <c r="CA1" s="64"/>
+      <c r="CB1" s="64"/>
+      <c r="CC1" s="64"/>
+      <c r="CD1" s="64"/>
+      <c r="CE1" s="64"/>
+      <c r="CF1" s="64"/>
+      <c r="CG1" s="64"/>
+      <c r="CH1" s="64"/>
+      <c r="CI1" s="64"/>
+      <c r="CJ1" s="64"/>
+      <c r="CK1" s="64"/>
+      <c r="CL1" s="64"/>
+      <c r="CM1" s="64"/>
+      <c r="CN1" s="64"/>
+      <c r="CO1" s="65"/>
+      <c r="CP1" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="CQ1" s="95"/>
-      <c r="CR1" s="95"/>
-      <c r="CS1" s="95"/>
-      <c r="CT1" s="95"/>
-      <c r="CU1" s="95"/>
-      <c r="CV1" s="95"/>
-      <c r="CW1" s="96"/>
-      <c r="CX1" s="100" t="s">
+      <c r="CQ1" s="67"/>
+      <c r="CR1" s="67"/>
+      <c r="CS1" s="67"/>
+      <c r="CT1" s="67"/>
+      <c r="CU1" s="67"/>
+      <c r="CV1" s="67"/>
+      <c r="CW1" s="68"/>
+      <c r="CX1" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="CY1" s="101"/>
-      <c r="CZ1" s="101"/>
-      <c r="DA1" s="101"/>
-      <c r="DB1" s="101"/>
-      <c r="DC1" s="101"/>
-      <c r="DD1" s="101"/>
-      <c r="DE1" s="101"/>
-      <c r="DF1" s="101"/>
-      <c r="DG1" s="101"/>
-      <c r="DH1" s="101"/>
-      <c r="DI1" s="101"/>
-      <c r="DJ1" s="101"/>
-      <c r="DK1" s="101"/>
-      <c r="DL1" s="101"/>
-      <c r="DM1" s="101"/>
-      <c r="DN1" s="101"/>
-      <c r="DO1" s="101"/>
-      <c r="DP1" s="101"/>
-      <c r="DQ1" s="101"/>
-      <c r="DR1" s="101"/>
-      <c r="DS1" s="101"/>
-      <c r="DT1" s="101"/>
-      <c r="DU1" s="101"/>
-      <c r="DV1" s="101"/>
-      <c r="DW1" s="101"/>
-      <c r="DX1" s="101"/>
-      <c r="DY1" s="101"/>
-      <c r="DZ1" s="101"/>
-      <c r="EA1" s="102"/>
-      <c r="EB1" s="71" t="s">
+      <c r="CY1" s="73"/>
+      <c r="CZ1" s="73"/>
+      <c r="DA1" s="73"/>
+      <c r="DB1" s="73"/>
+      <c r="DC1" s="73"/>
+      <c r="DD1" s="73"/>
+      <c r="DE1" s="73"/>
+      <c r="DF1" s="73"/>
+      <c r="DG1" s="73"/>
+      <c r="DH1" s="73"/>
+      <c r="DI1" s="73"/>
+      <c r="DJ1" s="73"/>
+      <c r="DK1" s="73"/>
+      <c r="DL1" s="73"/>
+      <c r="DM1" s="73"/>
+      <c r="DN1" s="73"/>
+      <c r="DO1" s="73"/>
+      <c r="DP1" s="73"/>
+      <c r="DQ1" s="73"/>
+      <c r="DR1" s="73"/>
+      <c r="DS1" s="73"/>
+      <c r="DT1" s="73"/>
+      <c r="DU1" s="73"/>
+      <c r="DV1" s="73"/>
+      <c r="DW1" s="73"/>
+      <c r="DX1" s="73"/>
+      <c r="DY1" s="73"/>
+      <c r="DZ1" s="73"/>
+      <c r="EA1" s="74"/>
+      <c r="EB1" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="EC1" s="71"/>
-      <c r="ED1" s="71"/>
-      <c r="EE1" s="71"/>
-      <c r="EF1" s="71"/>
-      <c r="EG1" s="71"/>
-      <c r="EH1" s="71"/>
-      <c r="EI1" s="71"/>
-      <c r="EJ1" s="71"/>
-      <c r="EK1" s="71"/>
-      <c r="EL1" s="71"/>
-      <c r="EM1" s="71"/>
-      <c r="EN1" s="71"/>
-      <c r="EO1" s="71"/>
-      <c r="EP1" s="71"/>
+      <c r="EC1" s="84"/>
+      <c r="ED1" s="84"/>
+      <c r="EE1" s="84"/>
+      <c r="EF1" s="84"/>
+      <c r="EG1" s="84"/>
+      <c r="EH1" s="84"/>
+      <c r="EI1" s="84"/>
+      <c r="EJ1" s="84"/>
+      <c r="EK1" s="84"/>
+      <c r="EL1" s="84"/>
+      <c r="EM1" s="84"/>
+      <c r="EN1" s="84"/>
+      <c r="EO1" s="84"/>
+      <c r="EP1" s="84"/>
     </row>
     <row r="2" spans="1:146" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="103" t="s">
+      <c r="A2" s="75" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="103" t="s">
+      <c r="B2" s="75" t="s">
         <v>124</v>
       </c>
       <c r="C2" s="76" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="103" t="s">
+      <c r="D2" s="75" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="66" t="s">
+      <c r="E2" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="66" t="s">
+      <c r="F2" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="66" t="s">
+      <c r="G2" s="77" t="s">
         <v>122</v>
       </c>
-      <c r="H2" s="66" t="s">
+      <c r="H2" s="77" t="s">
         <v>121</v>
       </c>
-      <c r="I2" s="72" t="s">
+      <c r="I2" s="85" t="s">
         <v>110</v>
       </c>
-      <c r="J2" s="73"/>
-      <c r="K2" s="74" t="s">
+      <c r="J2" s="86"/>
+      <c r="K2" s="87" t="s">
         <v>111</v>
       </c>
-      <c r="L2" s="75"/>
-      <c r="M2" s="66" t="s">
+      <c r="L2" s="88"/>
+      <c r="M2" s="77" t="s">
         <v>126</v>
       </c>
       <c r="N2" s="76" t="s">
@@ -2413,176 +2416,176 @@
       <c r="P2" s="76" t="s">
         <v>112</v>
       </c>
-      <c r="Q2" s="77" t="s">
+      <c r="Q2" s="89" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="77"/>
-      <c r="S2" s="77"/>
-      <c r="T2" s="77"/>
-      <c r="U2" s="77"/>
-      <c r="V2" s="77"/>
-      <c r="W2" s="77"/>
-      <c r="X2" s="78" t="s">
+      <c r="R2" s="89"/>
+      <c r="S2" s="89"/>
+      <c r="T2" s="89"/>
+      <c r="U2" s="89"/>
+      <c r="V2" s="89"/>
+      <c r="W2" s="89"/>
+      <c r="X2" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="Y2" s="78"/>
-      <c r="Z2" s="78"/>
-      <c r="AA2" s="78"/>
-      <c r="AB2" s="79" t="s">
+      <c r="Y2" s="90"/>
+      <c r="Z2" s="90"/>
+      <c r="AA2" s="90"/>
+      <c r="AB2" s="91" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="79"/>
-      <c r="AD2" s="79"/>
-      <c r="AE2" s="79"/>
-      <c r="AF2" s="79"/>
-      <c r="AG2" s="79"/>
-      <c r="AH2" s="79"/>
-      <c r="AI2" s="79"/>
-      <c r="AJ2" s="79"/>
-      <c r="AK2" s="80" t="s">
-        <v>16</v>
-      </c>
-      <c r="AL2" s="80"/>
-      <c r="AM2" s="80"/>
-      <c r="AN2" s="80"/>
-      <c r="AO2" s="80"/>
-      <c r="AP2" s="80"/>
-      <c r="AQ2" s="81" t="s">
+      <c r="AC2" s="91"/>
+      <c r="AD2" s="91"/>
+      <c r="AE2" s="91"/>
+      <c r="AF2" s="91"/>
+      <c r="AG2" s="91"/>
+      <c r="AH2" s="91"/>
+      <c r="AI2" s="91"/>
+      <c r="AJ2" s="91"/>
+      <c r="AK2" s="92" t="s">
+        <v>257</v>
+      </c>
+      <c r="AL2" s="92"/>
+      <c r="AM2" s="92"/>
+      <c r="AN2" s="92"/>
+      <c r="AO2" s="92"/>
+      <c r="AP2" s="92"/>
+      <c r="AQ2" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="AR2" s="81"/>
-      <c r="AS2" s="81"/>
-      <c r="AT2" s="81"/>
-      <c r="AU2" s="81"/>
-      <c r="AV2" s="81"/>
-      <c r="AW2" s="81"/>
-      <c r="AX2" s="81"/>
-      <c r="AY2" s="81"/>
-      <c r="AZ2" s="81"/>
-      <c r="BA2" s="81"/>
-      <c r="BB2" s="81"/>
-      <c r="BC2" s="81"/>
-      <c r="BD2" s="81"/>
-      <c r="BE2" s="81"/>
-      <c r="BF2" s="81"/>
-      <c r="BG2" s="81"/>
-      <c r="BH2" s="81"/>
-      <c r="BI2" s="81"/>
-      <c r="BJ2" s="81"/>
-      <c r="BK2" s="81"/>
-      <c r="BL2" s="81"/>
-      <c r="BM2" s="81"/>
-      <c r="BN2" s="82" t="s">
+      <c r="AR2" s="93"/>
+      <c r="AS2" s="93"/>
+      <c r="AT2" s="93"/>
+      <c r="AU2" s="93"/>
+      <c r="AV2" s="93"/>
+      <c r="AW2" s="93"/>
+      <c r="AX2" s="93"/>
+      <c r="AY2" s="93"/>
+      <c r="AZ2" s="93"/>
+      <c r="BA2" s="93"/>
+      <c r="BB2" s="93"/>
+      <c r="BC2" s="93"/>
+      <c r="BD2" s="93"/>
+      <c r="BE2" s="93"/>
+      <c r="BF2" s="93"/>
+      <c r="BG2" s="93"/>
+      <c r="BH2" s="93"/>
+      <c r="BI2" s="93"/>
+      <c r="BJ2" s="93"/>
+      <c r="BK2" s="93"/>
+      <c r="BL2" s="93"/>
+      <c r="BM2" s="93"/>
+      <c r="BN2" s="94" t="s">
         <v>18</v>
       </c>
-      <c r="BO2" s="82"/>
-      <c r="BP2" s="82"/>
-      <c r="BQ2" s="82"/>
-      <c r="BR2" s="82"/>
-      <c r="BS2" s="82"/>
-      <c r="BT2" s="82"/>
-      <c r="BU2" s="82"/>
-      <c r="BV2" s="82"/>
-      <c r="BW2" s="82"/>
-      <c r="BX2" s="82"/>
-      <c r="BY2" s="82"/>
-      <c r="BZ2" s="82"/>
-      <c r="CA2" s="82"/>
-      <c r="CB2" s="82"/>
-      <c r="CC2" s="82"/>
-      <c r="CD2" s="82"/>
-      <c r="CE2" s="82"/>
-      <c r="CF2" s="83" t="s">
+      <c r="BO2" s="94"/>
+      <c r="BP2" s="94"/>
+      <c r="BQ2" s="94"/>
+      <c r="BR2" s="94"/>
+      <c r="BS2" s="94"/>
+      <c r="BT2" s="94"/>
+      <c r="BU2" s="94"/>
+      <c r="BV2" s="94"/>
+      <c r="BW2" s="94"/>
+      <c r="BX2" s="94"/>
+      <c r="BY2" s="94"/>
+      <c r="BZ2" s="94"/>
+      <c r="CA2" s="94"/>
+      <c r="CB2" s="94"/>
+      <c r="CC2" s="94"/>
+      <c r="CD2" s="94"/>
+      <c r="CE2" s="94"/>
+      <c r="CF2" s="95" t="s">
         <v>19</v>
       </c>
-      <c r="CG2" s="83"/>
-      <c r="CH2" s="83"/>
-      <c r="CI2" s="77" t="s">
+      <c r="CG2" s="95"/>
+      <c r="CH2" s="95"/>
+      <c r="CI2" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="CJ2" s="77"/>
-      <c r="CK2" s="77"/>
-      <c r="CL2" s="77"/>
-      <c r="CM2" s="77"/>
-      <c r="CN2" s="77"/>
-      <c r="CO2" s="77"/>
-      <c r="CP2" s="97"/>
-      <c r="CQ2" s="98"/>
-      <c r="CR2" s="98"/>
-      <c r="CS2" s="98"/>
-      <c r="CT2" s="98"/>
-      <c r="CU2" s="98"/>
-      <c r="CV2" s="98"/>
-      <c r="CW2" s="99"/>
-      <c r="CX2" s="107" t="s">
+      <c r="CJ2" s="89"/>
+      <c r="CK2" s="89"/>
+      <c r="CL2" s="89"/>
+      <c r="CM2" s="89"/>
+      <c r="CN2" s="89"/>
+      <c r="CO2" s="89"/>
+      <c r="CP2" s="69"/>
+      <c r="CQ2" s="70"/>
+      <c r="CR2" s="70"/>
+      <c r="CS2" s="70"/>
+      <c r="CT2" s="70"/>
+      <c r="CU2" s="70"/>
+      <c r="CV2" s="70"/>
+      <c r="CW2" s="71"/>
+      <c r="CX2" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="CY2" s="67" t="s">
+      <c r="CY2" s="106" t="s">
         <v>22</v>
       </c>
-      <c r="CZ2" s="68"/>
-      <c r="DA2" s="68"/>
-      <c r="DB2" s="68"/>
-      <c r="DC2" s="68"/>
-      <c r="DD2" s="69"/>
-      <c r="DE2" s="84" t="s">
+      <c r="CZ2" s="107"/>
+      <c r="DA2" s="107"/>
+      <c r="DB2" s="107"/>
+      <c r="DC2" s="107"/>
+      <c r="DD2" s="108"/>
+      <c r="DE2" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="DF2" s="84"/>
-      <c r="DG2" s="84"/>
-      <c r="DH2" s="84"/>
-      <c r="DI2" s="84"/>
-      <c r="DJ2" s="84"/>
-      <c r="DK2" s="84"/>
-      <c r="DL2" s="84"/>
-      <c r="DM2" s="84"/>
-      <c r="DN2" s="84"/>
-      <c r="DO2" s="84"/>
-      <c r="DP2" s="104" t="s">
+      <c r="DF2" s="96"/>
+      <c r="DG2" s="96"/>
+      <c r="DH2" s="96"/>
+      <c r="DI2" s="96"/>
+      <c r="DJ2" s="96"/>
+      <c r="DK2" s="96"/>
+      <c r="DL2" s="96"/>
+      <c r="DM2" s="96"/>
+      <c r="DN2" s="96"/>
+      <c r="DO2" s="96"/>
+      <c r="DP2" s="78" t="s">
         <v>24</v>
       </c>
-      <c r="DQ2" s="105"/>
-      <c r="DR2" s="105"/>
-      <c r="DS2" s="105"/>
-      <c r="DT2" s="105"/>
-      <c r="DU2" s="105"/>
-      <c r="DV2" s="105"/>
-      <c r="DW2" s="105"/>
-      <c r="DX2" s="105"/>
-      <c r="DY2" s="105"/>
-      <c r="DZ2" s="105"/>
-      <c r="EA2" s="106"/>
+      <c r="DQ2" s="79"/>
+      <c r="DR2" s="79"/>
+      <c r="DS2" s="79"/>
+      <c r="DT2" s="79"/>
+      <c r="DU2" s="79"/>
+      <c r="DV2" s="79"/>
+      <c r="DW2" s="79"/>
+      <c r="DX2" s="79"/>
+      <c r="DY2" s="79"/>
+      <c r="DZ2" s="79"/>
+      <c r="EA2" s="80"/>
       <c r="EB2" s="36"/>
       <c r="EC2" s="36"/>
       <c r="ED2" s="36"/>
       <c r="EE2" s="36"/>
-      <c r="EF2" s="63" t="s">
+      <c r="EF2" s="103" t="s">
         <v>25</v>
       </c>
-      <c r="EG2" s="64"/>
-      <c r="EH2" s="64"/>
-      <c r="EI2" s="65"/>
-      <c r="EJ2" s="85" t="s">
+      <c r="EG2" s="104"/>
+      <c r="EH2" s="104"/>
+      <c r="EI2" s="105"/>
+      <c r="EJ2" s="97" t="s">
         <v>26</v>
       </c>
-      <c r="EK2" s="86"/>
-      <c r="EL2" s="86"/>
-      <c r="EM2" s="86"/>
-      <c r="EN2" s="87"/>
-      <c r="EO2" s="70" t="s">
+      <c r="EK2" s="98"/>
+      <c r="EL2" s="98"/>
+      <c r="EM2" s="98"/>
+      <c r="EN2" s="99"/>
+      <c r="EO2" s="83" t="s">
         <v>106</v>
       </c>
-      <c r="EP2" s="70"/>
+      <c r="EP2" s="83"/>
     </row>
     <row r="3" spans="1:146" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
       <c r="B3" s="76"/>
       <c r="C3" s="76"/>
       <c r="D3" s="76"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
       <c r="I3" s="34" t="s">
         <v>8</v>
       </c>
@@ -2595,7 +2598,7 @@
       <c r="L3" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="66"/>
+      <c r="M3" s="77"/>
       <c r="N3" s="76"/>
       <c r="O3" s="76"/>
       <c r="P3" s="76"/>
@@ -2854,7 +2857,7 @@
       <c r="CW3" s="52" t="s">
         <v>70</v>
       </c>
-      <c r="CX3" s="108"/>
+      <c r="CX3" s="82"/>
       <c r="CY3" s="53" t="s">
         <v>71</v>
       </c>
@@ -33166,19 +33169,11 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="Q1:CO1"/>
-    <mergeCell ref="CP1:CW2"/>
-    <mergeCell ref="CX1:EA1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="DP2:EA2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="CX2:CX3"/>
+    <mergeCell ref="EF2:EI2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="CY2:DD2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="G2:G3"/>
     <mergeCell ref="EO2:EP2"/>
     <mergeCell ref="EB1:EP1"/>
     <mergeCell ref="I2:J2"/>
@@ -33195,13 +33190,21 @@
     <mergeCell ref="DE2:DO2"/>
     <mergeCell ref="EJ2:EN2"/>
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="EF2:EI2"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="CY2:DD2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="Q1:CO1"/>
+    <mergeCell ref="CP1:CW2"/>
+    <mergeCell ref="CX1:EA1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="DP2:EA2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="CX2:CX3"/>
   </mergeCells>
-  <dataValidations xWindow="246" yWindow="503" count="7">
+  <dataValidations xWindow="246" yWindow="503" count="11">
     <dataValidation type="list" allowBlank="1" sqref="A3" xr:uid="{C94C9C08-E811-49C1-A6EE-6ABF7BB7DF7D}">
       <formula1>"Stt5_Xeôtô,Stt6_Phươngtiệnvậntảikhác,Stt7_Máymócthiếtbị,Stt9_Tàisảncốđịnhhữuhìnhkhác,Stt10_Quyềnsửdụngđất,Stt8_Câylâunămsúcvậtlàmviệc,Stt4_Vậtkiếntrúc,Stt3_Nhàcôngtrìnhxâydựng"</formula1>
     </dataValidation>
@@ -33217,8 +33220,12 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Vui lòng chọn cách tính khấu hao,hao mòn: Tính khấu hao, Tính hao mòn, Tính cả hai" sqref="EB4:EB2188" xr:uid="{B12539CD-C7F9-4B49-9682-74888345B2FA}">
       <formula1>"---, Tính khấu hao, Tính hao mòn, Tính cả hai"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Vui lòng nhập ngày tháng theo định dạng dd/mm/yyyy. Ví dụ: 30/04/2011" sqref="BF4:BF2184 BY4:BY2184 DR4:DR2184 DT4:DT2184 DV4:DV2184 DX4:DX2184 DZ4:DZ2184 EC4:EF2184 EI4:EJ2184 CR4:CR2183" xr:uid="{47DCBA19-C5A7-4862-B806-68E4E8267070}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Vui lòng nhập ngày tháng theo định dạng dd/mm/yyyy. Ví dụ: 30/04/2011" sqref="BF4:BF2184 BY4:BY2184 DR4:DR2184 DT4:DT2184 DV4:DV2184 DX4:DX2184 DZ4:DZ2184 EC4:EF2184 EI4:EJ2184 CR4:CR2183 CS4:CS2191" xr:uid="{47DCBA19-C5A7-4862-B806-68E4E8267070}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Nguồn Hình Thành" prompt="Vui lòng sang bên Sheet Huongdannhapthongtin để xem danh sách các nguồn hình thành và nhập theo định dạng:_x000a_Nguồn A;Nguồn B;Nguồn C;..." sqref="N4:N2186" xr:uid="{D7602B7F-E27A-4FFA-8FC7-3E6F3D99FD59}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Điền giá trị tương ứng với mỗi nguồn hình thành đã nhập. Vui lòng nhập theo định dạng: Giá trị A;Giá trị B;.... Ví dụ: 200000;300000;100000" sqref="O4:O2201" xr:uid="{0AB25960-CA5D-42F7-81D2-6312F02733A6}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Nhập giá trị thuế được miễn nếu chọn Có &quot;Được miễn thuế&quot;" sqref="AR4:AR2191" xr:uid="{03813426-80C0-4F72-9E18-DDA4EFF0FD07}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Chọn tài sản khuôn viên đất nếu tài sản Nhà &quot;có quản lý đất&quot;" sqref="AC4:AC2123" xr:uid="{7FDFD0B1-29CE-4007-9B42-A8254A37B205}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Chọn khuôn viên đất nếu Vật kiến trúc thuộc khuôn viên nào đó" sqref="AK4:AK2047" xr:uid="{D8CA720F-0AA0-424C-8580-5622EA4C7559}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -33285,378 +33292,378 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:146" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="109" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="135"/>
-      <c r="F1" s="135"/>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="135"/>
-      <c r="L1" s="135"/>
-      <c r="M1" s="135"/>
-      <c r="N1" s="135"/>
-      <c r="O1" s="135"/>
-      <c r="P1" s="136"/>
-      <c r="Q1" s="137" t="s">
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="111"/>
+      <c r="Q1" s="112" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="138"/>
-      <c r="S1" s="138"/>
-      <c r="T1" s="138"/>
-      <c r="U1" s="138"/>
-      <c r="V1" s="138"/>
-      <c r="W1" s="138"/>
-      <c r="X1" s="138"/>
-      <c r="Y1" s="138"/>
-      <c r="Z1" s="138"/>
-      <c r="AA1" s="138"/>
-      <c r="AB1" s="138"/>
-      <c r="AC1" s="138"/>
-      <c r="AD1" s="138"/>
-      <c r="AE1" s="138"/>
-      <c r="AF1" s="138"/>
-      <c r="AG1" s="138"/>
-      <c r="AH1" s="138"/>
-      <c r="AI1" s="138"/>
-      <c r="AJ1" s="138"/>
-      <c r="AK1" s="138"/>
-      <c r="AL1" s="138"/>
-      <c r="AM1" s="138"/>
-      <c r="AN1" s="138"/>
-      <c r="AO1" s="138"/>
-      <c r="AP1" s="138"/>
-      <c r="AQ1" s="138"/>
-      <c r="AR1" s="138"/>
-      <c r="AS1" s="138"/>
-      <c r="AT1" s="138"/>
-      <c r="AU1" s="138"/>
-      <c r="AV1" s="138"/>
-      <c r="AW1" s="138"/>
-      <c r="AX1" s="138"/>
-      <c r="AY1" s="138"/>
-      <c r="AZ1" s="138"/>
-      <c r="BA1" s="138"/>
-      <c r="BB1" s="138"/>
-      <c r="BC1" s="138"/>
-      <c r="BD1" s="138"/>
-      <c r="BE1" s="138"/>
-      <c r="BF1" s="138"/>
-      <c r="BG1" s="138"/>
-      <c r="BH1" s="138"/>
-      <c r="BI1" s="138"/>
-      <c r="BJ1" s="138"/>
-      <c r="BK1" s="138"/>
-      <c r="BL1" s="138"/>
-      <c r="BM1" s="138"/>
-      <c r="BN1" s="138"/>
-      <c r="BO1" s="138"/>
-      <c r="BP1" s="138"/>
-      <c r="BQ1" s="138"/>
-      <c r="BR1" s="138"/>
-      <c r="BS1" s="138"/>
-      <c r="BT1" s="138"/>
-      <c r="BU1" s="138"/>
-      <c r="BV1" s="138"/>
-      <c r="BW1" s="138"/>
-      <c r="BX1" s="138"/>
-      <c r="BY1" s="138"/>
-      <c r="BZ1" s="138"/>
-      <c r="CA1" s="138"/>
-      <c r="CB1" s="138"/>
-      <c r="CC1" s="138"/>
-      <c r="CD1" s="138"/>
-      <c r="CE1" s="138"/>
-      <c r="CF1" s="138"/>
-      <c r="CG1" s="138"/>
-      <c r="CH1" s="138"/>
-      <c r="CI1" s="138"/>
-      <c r="CJ1" s="138"/>
-      <c r="CK1" s="138"/>
-      <c r="CL1" s="138"/>
-      <c r="CM1" s="138"/>
-      <c r="CN1" s="138"/>
-      <c r="CO1" s="139"/>
-      <c r="CP1" s="140" t="s">
+      <c r="R1" s="113"/>
+      <c r="S1" s="113"/>
+      <c r="T1" s="113"/>
+      <c r="U1" s="113"/>
+      <c r="V1" s="113"/>
+      <c r="W1" s="113"/>
+      <c r="X1" s="113"/>
+      <c r="Y1" s="113"/>
+      <c r="Z1" s="113"/>
+      <c r="AA1" s="113"/>
+      <c r="AB1" s="113"/>
+      <c r="AC1" s="113"/>
+      <c r="AD1" s="113"/>
+      <c r="AE1" s="113"/>
+      <c r="AF1" s="113"/>
+      <c r="AG1" s="113"/>
+      <c r="AH1" s="113"/>
+      <c r="AI1" s="113"/>
+      <c r="AJ1" s="113"/>
+      <c r="AK1" s="113"/>
+      <c r="AL1" s="113"/>
+      <c r="AM1" s="113"/>
+      <c r="AN1" s="113"/>
+      <c r="AO1" s="113"/>
+      <c r="AP1" s="113"/>
+      <c r="AQ1" s="113"/>
+      <c r="AR1" s="113"/>
+      <c r="AS1" s="113"/>
+      <c r="AT1" s="113"/>
+      <c r="AU1" s="113"/>
+      <c r="AV1" s="113"/>
+      <c r="AW1" s="113"/>
+      <c r="AX1" s="113"/>
+      <c r="AY1" s="113"/>
+      <c r="AZ1" s="113"/>
+      <c r="BA1" s="113"/>
+      <c r="BB1" s="113"/>
+      <c r="BC1" s="113"/>
+      <c r="BD1" s="113"/>
+      <c r="BE1" s="113"/>
+      <c r="BF1" s="113"/>
+      <c r="BG1" s="113"/>
+      <c r="BH1" s="113"/>
+      <c r="BI1" s="113"/>
+      <c r="BJ1" s="113"/>
+      <c r="BK1" s="113"/>
+      <c r="BL1" s="113"/>
+      <c r="BM1" s="113"/>
+      <c r="BN1" s="113"/>
+      <c r="BO1" s="113"/>
+      <c r="BP1" s="113"/>
+      <c r="BQ1" s="113"/>
+      <c r="BR1" s="113"/>
+      <c r="BS1" s="113"/>
+      <c r="BT1" s="113"/>
+      <c r="BU1" s="113"/>
+      <c r="BV1" s="113"/>
+      <c r="BW1" s="113"/>
+      <c r="BX1" s="113"/>
+      <c r="BY1" s="113"/>
+      <c r="BZ1" s="113"/>
+      <c r="CA1" s="113"/>
+      <c r="CB1" s="113"/>
+      <c r="CC1" s="113"/>
+      <c r="CD1" s="113"/>
+      <c r="CE1" s="113"/>
+      <c r="CF1" s="113"/>
+      <c r="CG1" s="113"/>
+      <c r="CH1" s="113"/>
+      <c r="CI1" s="113"/>
+      <c r="CJ1" s="113"/>
+      <c r="CK1" s="113"/>
+      <c r="CL1" s="113"/>
+      <c r="CM1" s="113"/>
+      <c r="CN1" s="113"/>
+      <c r="CO1" s="114"/>
+      <c r="CP1" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="CQ1" s="141"/>
-      <c r="CR1" s="141"/>
-      <c r="CS1" s="141"/>
-      <c r="CT1" s="141"/>
-      <c r="CU1" s="141"/>
-      <c r="CV1" s="141"/>
-      <c r="CW1" s="142"/>
-      <c r="CX1" s="146" t="s">
+      <c r="CQ1" s="116"/>
+      <c r="CR1" s="116"/>
+      <c r="CS1" s="116"/>
+      <c r="CT1" s="116"/>
+      <c r="CU1" s="116"/>
+      <c r="CV1" s="116"/>
+      <c r="CW1" s="117"/>
+      <c r="CX1" s="121" t="s">
         <v>3</v>
       </c>
-      <c r="CY1" s="147"/>
-      <c r="CZ1" s="147"/>
-      <c r="DA1" s="147"/>
-      <c r="DB1" s="147"/>
-      <c r="DC1" s="147"/>
-      <c r="DD1" s="147"/>
-      <c r="DE1" s="147"/>
-      <c r="DF1" s="147"/>
-      <c r="DG1" s="147"/>
-      <c r="DH1" s="147"/>
-      <c r="DI1" s="147"/>
-      <c r="DJ1" s="147"/>
-      <c r="DK1" s="147"/>
-      <c r="DL1" s="147"/>
-      <c r="DM1" s="147"/>
-      <c r="DN1" s="147"/>
-      <c r="DO1" s="147"/>
-      <c r="DP1" s="147"/>
-      <c r="DQ1" s="147"/>
-      <c r="DR1" s="147"/>
-      <c r="DS1" s="147"/>
-      <c r="DT1" s="147"/>
-      <c r="DU1" s="147"/>
-      <c r="DV1" s="147"/>
-      <c r="DW1" s="147"/>
-      <c r="DX1" s="147"/>
-      <c r="DY1" s="147"/>
-      <c r="DZ1" s="147"/>
-      <c r="EA1" s="148"/>
-      <c r="EB1" s="149" t="s">
+      <c r="CY1" s="122"/>
+      <c r="CZ1" s="122"/>
+      <c r="DA1" s="122"/>
+      <c r="DB1" s="122"/>
+      <c r="DC1" s="122"/>
+      <c r="DD1" s="122"/>
+      <c r="DE1" s="122"/>
+      <c r="DF1" s="122"/>
+      <c r="DG1" s="122"/>
+      <c r="DH1" s="122"/>
+      <c r="DI1" s="122"/>
+      <c r="DJ1" s="122"/>
+      <c r="DK1" s="122"/>
+      <c r="DL1" s="122"/>
+      <c r="DM1" s="122"/>
+      <c r="DN1" s="122"/>
+      <c r="DO1" s="122"/>
+      <c r="DP1" s="122"/>
+      <c r="DQ1" s="122"/>
+      <c r="DR1" s="122"/>
+      <c r="DS1" s="122"/>
+      <c r="DT1" s="122"/>
+      <c r="DU1" s="122"/>
+      <c r="DV1" s="122"/>
+      <c r="DW1" s="122"/>
+      <c r="DX1" s="122"/>
+      <c r="DY1" s="122"/>
+      <c r="DZ1" s="122"/>
+      <c r="EA1" s="123"/>
+      <c r="EB1" s="124" t="s">
         <v>4</v>
       </c>
-      <c r="EC1" s="149"/>
-      <c r="ED1" s="149"/>
-      <c r="EE1" s="149"/>
-      <c r="EF1" s="149"/>
-      <c r="EG1" s="149"/>
-      <c r="EH1" s="149"/>
-      <c r="EI1" s="149"/>
-      <c r="EJ1" s="149"/>
-      <c r="EK1" s="149"/>
-      <c r="EL1" s="149"/>
-      <c r="EM1" s="149"/>
-      <c r="EN1" s="149"/>
-      <c r="EO1" s="149"/>
-      <c r="EP1" s="149"/>
+      <c r="EC1" s="124"/>
+      <c r="ED1" s="124"/>
+      <c r="EE1" s="124"/>
+      <c r="EF1" s="124"/>
+      <c r="EG1" s="124"/>
+      <c r="EH1" s="124"/>
+      <c r="EI1" s="124"/>
+      <c r="EJ1" s="124"/>
+      <c r="EK1" s="124"/>
+      <c r="EL1" s="124"/>
+      <c r="EM1" s="124"/>
+      <c r="EN1" s="124"/>
+      <c r="EO1" s="124"/>
+      <c r="EP1" s="124"/>
     </row>
     <row r="2" spans="1:146" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="150" t="s">
+      <c r="A2" s="125" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="150" t="s">
+      <c r="B2" s="125" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="132" t="s">
+      <c r="C2" s="127" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="150" t="s">
+      <c r="D2" s="125" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="130" t="s">
+      <c r="E2" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="130" t="s">
+      <c r="F2" s="128" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="130" t="s">
+      <c r="G2" s="128" t="s">
         <v>122</v>
       </c>
-      <c r="H2" s="130" t="s">
+      <c r="H2" s="128" t="s">
         <v>121</v>
       </c>
-      <c r="I2" s="152" t="s">
+      <c r="I2" s="131" t="s">
         <v>110</v>
       </c>
-      <c r="J2" s="153"/>
-      <c r="K2" s="154" t="s">
+      <c r="J2" s="132"/>
+      <c r="K2" s="133" t="s">
         <v>111</v>
       </c>
-      <c r="L2" s="155"/>
-      <c r="M2" s="130" t="s">
+      <c r="L2" s="134"/>
+      <c r="M2" s="128" t="s">
         <v>126</v>
       </c>
-      <c r="N2" s="132" t="s">
+      <c r="N2" s="127" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="132" t="s">
+      <c r="O2" s="127" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="132" t="s">
+      <c r="P2" s="127" t="s">
         <v>112</v>
       </c>
-      <c r="Q2" s="115" t="s">
+      <c r="Q2" s="135" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="115"/>
-      <c r="S2" s="115"/>
-      <c r="T2" s="115"/>
-      <c r="U2" s="115"/>
-      <c r="V2" s="115"/>
-      <c r="W2" s="115"/>
-      <c r="X2" s="109" t="s">
+      <c r="R2" s="135"/>
+      <c r="S2" s="135"/>
+      <c r="T2" s="135"/>
+      <c r="U2" s="135"/>
+      <c r="V2" s="135"/>
+      <c r="W2" s="135"/>
+      <c r="X2" s="136" t="s">
         <v>14</v>
       </c>
-      <c r="Y2" s="109"/>
-      <c r="Z2" s="109"/>
-      <c r="AA2" s="109"/>
-      <c r="AB2" s="151" t="s">
+      <c r="Y2" s="136"/>
+      <c r="Z2" s="136"/>
+      <c r="AA2" s="136"/>
+      <c r="AB2" s="130" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="151"/>
-      <c r="AD2" s="151"/>
-      <c r="AE2" s="151"/>
-      <c r="AF2" s="151"/>
-      <c r="AG2" s="151"/>
-      <c r="AH2" s="151"/>
-      <c r="AI2" s="151"/>
-      <c r="AJ2" s="151"/>
-      <c r="AK2" s="111" t="s">
+      <c r="AC2" s="130"/>
+      <c r="AD2" s="130"/>
+      <c r="AE2" s="130"/>
+      <c r="AF2" s="130"/>
+      <c r="AG2" s="130"/>
+      <c r="AH2" s="130"/>
+      <c r="AI2" s="130"/>
+      <c r="AJ2" s="130"/>
+      <c r="AK2" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="AL2" s="111"/>
-      <c r="AM2" s="111"/>
-      <c r="AN2" s="111"/>
-      <c r="AO2" s="111"/>
-      <c r="AP2" s="111"/>
-      <c r="AQ2" s="112" t="s">
+      <c r="AL2" s="138"/>
+      <c r="AM2" s="138"/>
+      <c r="AN2" s="138"/>
+      <c r="AO2" s="138"/>
+      <c r="AP2" s="138"/>
+      <c r="AQ2" s="139" t="s">
         <v>17</v>
       </c>
-      <c r="AR2" s="112"/>
-      <c r="AS2" s="112"/>
-      <c r="AT2" s="112"/>
-      <c r="AU2" s="112"/>
-      <c r="AV2" s="112"/>
-      <c r="AW2" s="112"/>
-      <c r="AX2" s="112"/>
-      <c r="AY2" s="112"/>
-      <c r="AZ2" s="112"/>
-      <c r="BA2" s="112"/>
-      <c r="BB2" s="112"/>
-      <c r="BC2" s="112"/>
-      <c r="BD2" s="112"/>
-      <c r="BE2" s="112"/>
-      <c r="BF2" s="112"/>
-      <c r="BG2" s="112"/>
-      <c r="BH2" s="112"/>
-      <c r="BI2" s="112"/>
-      <c r="BJ2" s="112"/>
-      <c r="BK2" s="112"/>
-      <c r="BL2" s="112"/>
-      <c r="BM2" s="112"/>
-      <c r="BN2" s="113" t="s">
+      <c r="AR2" s="139"/>
+      <c r="AS2" s="139"/>
+      <c r="AT2" s="139"/>
+      <c r="AU2" s="139"/>
+      <c r="AV2" s="139"/>
+      <c r="AW2" s="139"/>
+      <c r="AX2" s="139"/>
+      <c r="AY2" s="139"/>
+      <c r="AZ2" s="139"/>
+      <c r="BA2" s="139"/>
+      <c r="BB2" s="139"/>
+      <c r="BC2" s="139"/>
+      <c r="BD2" s="139"/>
+      <c r="BE2" s="139"/>
+      <c r="BF2" s="139"/>
+      <c r="BG2" s="139"/>
+      <c r="BH2" s="139"/>
+      <c r="BI2" s="139"/>
+      <c r="BJ2" s="139"/>
+      <c r="BK2" s="139"/>
+      <c r="BL2" s="139"/>
+      <c r="BM2" s="139"/>
+      <c r="BN2" s="140" t="s">
         <v>18</v>
       </c>
-      <c r="BO2" s="113"/>
-      <c r="BP2" s="113"/>
-      <c r="BQ2" s="113"/>
-      <c r="BR2" s="113"/>
-      <c r="BS2" s="113"/>
-      <c r="BT2" s="113"/>
-      <c r="BU2" s="113"/>
-      <c r="BV2" s="113"/>
-      <c r="BW2" s="113"/>
-      <c r="BX2" s="113"/>
-      <c r="BY2" s="113"/>
-      <c r="BZ2" s="113"/>
-      <c r="CA2" s="113"/>
-      <c r="CB2" s="113"/>
-      <c r="CC2" s="113"/>
-      <c r="CD2" s="113"/>
-      <c r="CE2" s="113"/>
-      <c r="CF2" s="114" t="s">
+      <c r="BO2" s="140"/>
+      <c r="BP2" s="140"/>
+      <c r="BQ2" s="140"/>
+      <c r="BR2" s="140"/>
+      <c r="BS2" s="140"/>
+      <c r="BT2" s="140"/>
+      <c r="BU2" s="140"/>
+      <c r="BV2" s="140"/>
+      <c r="BW2" s="140"/>
+      <c r="BX2" s="140"/>
+      <c r="BY2" s="140"/>
+      <c r="BZ2" s="140"/>
+      <c r="CA2" s="140"/>
+      <c r="CB2" s="140"/>
+      <c r="CC2" s="140"/>
+      <c r="CD2" s="140"/>
+      <c r="CE2" s="140"/>
+      <c r="CF2" s="141" t="s">
         <v>19</v>
       </c>
-      <c r="CG2" s="114"/>
-      <c r="CH2" s="114"/>
-      <c r="CI2" s="115" t="s">
+      <c r="CG2" s="141"/>
+      <c r="CH2" s="141"/>
+      <c r="CI2" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="CJ2" s="115"/>
-      <c r="CK2" s="115"/>
-      <c r="CL2" s="115"/>
-      <c r="CM2" s="115"/>
-      <c r="CN2" s="115"/>
-      <c r="CO2" s="115"/>
-      <c r="CP2" s="143"/>
-      <c r="CQ2" s="144"/>
-      <c r="CR2" s="144"/>
-      <c r="CS2" s="144"/>
-      <c r="CT2" s="144"/>
-      <c r="CU2" s="144"/>
-      <c r="CV2" s="144"/>
-      <c r="CW2" s="145"/>
-      <c r="CX2" s="116" t="s">
+      <c r="CJ2" s="135"/>
+      <c r="CK2" s="135"/>
+      <c r="CL2" s="135"/>
+      <c r="CM2" s="135"/>
+      <c r="CN2" s="135"/>
+      <c r="CO2" s="135"/>
+      <c r="CP2" s="118"/>
+      <c r="CQ2" s="119"/>
+      <c r="CR2" s="119"/>
+      <c r="CS2" s="119"/>
+      <c r="CT2" s="119"/>
+      <c r="CU2" s="119"/>
+      <c r="CV2" s="119"/>
+      <c r="CW2" s="120"/>
+      <c r="CX2" s="142" t="s">
         <v>21</v>
       </c>
-      <c r="CY2" s="118" t="s">
+      <c r="CY2" s="144" t="s">
         <v>22</v>
       </c>
-      <c r="CZ2" s="119"/>
-      <c r="DA2" s="119"/>
-      <c r="DB2" s="119"/>
-      <c r="DC2" s="119"/>
-      <c r="DD2" s="120"/>
-      <c r="DE2" s="84" t="s">
+      <c r="CZ2" s="145"/>
+      <c r="DA2" s="145"/>
+      <c r="DB2" s="145"/>
+      <c r="DC2" s="145"/>
+      <c r="DD2" s="146"/>
+      <c r="DE2" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="DF2" s="84"/>
-      <c r="DG2" s="84"/>
-      <c r="DH2" s="84"/>
-      <c r="DI2" s="84"/>
-      <c r="DJ2" s="84"/>
-      <c r="DK2" s="84"/>
-      <c r="DL2" s="84"/>
-      <c r="DM2" s="84"/>
-      <c r="DN2" s="84"/>
-      <c r="DO2" s="84"/>
-      <c r="DP2" s="121" t="s">
+      <c r="DF2" s="96"/>
+      <c r="DG2" s="96"/>
+      <c r="DH2" s="96"/>
+      <c r="DI2" s="96"/>
+      <c r="DJ2" s="96"/>
+      <c r="DK2" s="96"/>
+      <c r="DL2" s="96"/>
+      <c r="DM2" s="96"/>
+      <c r="DN2" s="96"/>
+      <c r="DO2" s="96"/>
+      <c r="DP2" s="147" t="s">
         <v>24</v>
       </c>
-      <c r="DQ2" s="122"/>
-      <c r="DR2" s="122"/>
-      <c r="DS2" s="122"/>
-      <c r="DT2" s="122"/>
-      <c r="DU2" s="122"/>
-      <c r="DV2" s="122"/>
-      <c r="DW2" s="122"/>
-      <c r="DX2" s="122"/>
-      <c r="DY2" s="122"/>
-      <c r="DZ2" s="122"/>
-      <c r="EA2" s="123"/>
+      <c r="DQ2" s="148"/>
+      <c r="DR2" s="148"/>
+      <c r="DS2" s="148"/>
+      <c r="DT2" s="148"/>
+      <c r="DU2" s="148"/>
+      <c r="DV2" s="148"/>
+      <c r="DW2" s="148"/>
+      <c r="DX2" s="148"/>
+      <c r="DY2" s="148"/>
+      <c r="DZ2" s="148"/>
+      <c r="EA2" s="149"/>
       <c r="EB2" s="1"/>
       <c r="EC2" s="1"/>
       <c r="ED2" s="1"/>
       <c r="EE2" s="1"/>
-      <c r="EF2" s="124" t="s">
+      <c r="EF2" s="150" t="s">
         <v>25</v>
       </c>
-      <c r="EG2" s="125"/>
-      <c r="EH2" s="125"/>
-      <c r="EI2" s="126"/>
-      <c r="EJ2" s="127" t="s">
+      <c r="EG2" s="151"/>
+      <c r="EH2" s="151"/>
+      <c r="EI2" s="152"/>
+      <c r="EJ2" s="153" t="s">
         <v>26</v>
       </c>
-      <c r="EK2" s="128"/>
-      <c r="EL2" s="128"/>
-      <c r="EM2" s="128"/>
-      <c r="EN2" s="129"/>
-      <c r="EO2" s="110" t="s">
+      <c r="EK2" s="154"/>
+      <c r="EL2" s="154"/>
+      <c r="EM2" s="154"/>
+      <c r="EN2" s="155"/>
+      <c r="EO2" s="137" t="s">
         <v>106</v>
       </c>
-      <c r="EP2" s="110"/>
+      <c r="EP2" s="137"/>
     </row>
     <row r="3" spans="1:146" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="133"/>
-      <c r="B3" s="133"/>
-      <c r="C3" s="133"/>
-      <c r="D3" s="133"/>
-      <c r="E3" s="131"/>
-      <c r="F3" s="131"/>
-      <c r="G3" s="131"/>
-      <c r="H3" s="131"/>
+      <c r="A3" s="126"/>
+      <c r="B3" s="126"/>
+      <c r="C3" s="126"/>
+      <c r="D3" s="126"/>
+      <c r="E3" s="129"/>
+      <c r="F3" s="129"/>
+      <c r="G3" s="129"/>
+      <c r="H3" s="129"/>
       <c r="I3" s="2" t="s">
         <v>8</v>
       </c>
@@ -33669,10 +33676,10 @@
       <c r="L3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="131"/>
-      <c r="N3" s="133"/>
-      <c r="O3" s="133"/>
-      <c r="P3" s="133"/>
+      <c r="M3" s="129"/>
+      <c r="N3" s="126"/>
+      <c r="O3" s="126"/>
+      <c r="P3" s="126"/>
       <c r="Q3" s="4" t="s">
         <v>27</v>
       </c>
@@ -33928,7 +33935,7 @@
       <c r="CW3" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="CX3" s="117"/>
+      <c r="CX3" s="143"/>
       <c r="CY3" s="21" t="s">
         <v>71</v>
       </c>
@@ -34523,6 +34530,24 @@
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="X2:AA2"/>
+    <mergeCell ref="EO2:EP2"/>
+    <mergeCell ref="AK2:AP2"/>
+    <mergeCell ref="AQ2:BM2"/>
+    <mergeCell ref="BN2:CE2"/>
+    <mergeCell ref="CF2:CH2"/>
+    <mergeCell ref="CI2:CO2"/>
+    <mergeCell ref="CX2:CX3"/>
+    <mergeCell ref="CY2:DD2"/>
+    <mergeCell ref="DE2:DO2"/>
+    <mergeCell ref="DP2:EA2"/>
+    <mergeCell ref="EF2:EI2"/>
+    <mergeCell ref="EJ2:EN2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:W2"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="Q1:CO1"/>
     <mergeCell ref="CP1:CW2"/>
@@ -34539,24 +34564,6 @@
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="K2:L2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:W2"/>
-    <mergeCell ref="X2:AA2"/>
-    <mergeCell ref="EO2:EP2"/>
-    <mergeCell ref="AK2:AP2"/>
-    <mergeCell ref="AQ2:BM2"/>
-    <mergeCell ref="BN2:CE2"/>
-    <mergeCell ref="CF2:CH2"/>
-    <mergeCell ref="CI2:CO2"/>
-    <mergeCell ref="CX2:CX3"/>
-    <mergeCell ref="CY2:DD2"/>
-    <mergeCell ref="DE2:DO2"/>
-    <mergeCell ref="DP2:EA2"/>
-    <mergeCell ref="EF2:EI2"/>
-    <mergeCell ref="EJ2:EN2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="B3" xr:uid="{ACD79C73-1AC5-4E5C-B174-8735C17FE353}">

</xml_diff>